<commit_message>
ID-100/121: fetch additional FHIR data and check coverage payer (#62)
* requirements planning tweak

* fetch coverage payor during hook processing

* capture Inferno organization id during registration

* check that the coverage payor id matches what indicated in registration and matches the CRD Organization profile

* check that additional data could be fetched during hook invocations

* add new tests to hook group

* update presets
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/hti-4/CRD 2.2.1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5E5900-ADE4-4945-BFF8-9B20BD1110FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D21B98DF-24F3-B743-A229-B31E36E95DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="320" yWindow="1280" windowWidth="34240" windowHeight="21260" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
+    <workbookView xWindow="320" yWindow="760" windowWidth="34240" windowHeight="21260" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="9" r:id="rId1"/>
@@ -3825,9 +3825,6 @@
     <t>Mechanical: require that FHIR API testing happen after hook invocations and include patients on which CRD was invoked so that Inferno can observe the persisted coverage-information extension</t>
   </si>
   <si>
-    <t>Mechanical: check for coverage-info across all responses (updated from 3 cards)</t>
-  </si>
-  <si>
     <t>Mechanical: check that the provided scopes match the expected scopes indicated by Inferno. (future - check that scopes are enforced)</t>
   </si>
   <si>
@@ -3892,6 +3889,9 @@
   </si>
   <si>
     <t>ID-110</t>
+  </si>
+  <si>
+    <t>Mechanical: check for coverage-info across all responses</t>
   </si>
 </sst>
 </file>
@@ -4804,6 +4804,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AF434"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4939,7 +4940,7 @@
       <c r="U2" s="27"/>
       <c r="Z2" s="28"/>
     </row>
-    <row r="3" spans="1:32" ht="34" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:32" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>94</v>
       </c>
@@ -4971,7 +4972,7 @@
       <c r="AE3" s="24"/>
       <c r="AF3" s="24"/>
     </row>
-    <row r="4" spans="1:32" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:32" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
         <v>98</v>
       </c>
@@ -5000,7 +5001,7 @@
       <c r="AA4" s="24"/>
       <c r="AB4" s="24"/>
     </row>
-    <row r="5" spans="1:32" ht="68" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:32" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="s">
         <v>101</v>
       </c>
@@ -5049,10 +5050,10 @@
         <v>807</v>
       </c>
       <c r="S6" s="27" t="s">
-        <v>820</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" ht="34" x14ac:dyDescent="0.2">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
         <v>106</v>
       </c>
@@ -5101,10 +5102,10 @@
         <v>808</v>
       </c>
       <c r="S8" s="27" t="s">
-        <v>821</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" ht="34" x14ac:dyDescent="0.2">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="25" t="s">
         <v>112</v>
       </c>
@@ -5127,7 +5128,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:32" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
         <v>115</v>
       </c>
@@ -5176,10 +5177,10 @@
         <v>82</v>
       </c>
       <c r="S11" s="27" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" ht="119" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="12" spans="1:32" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="s">
         <v>122</v>
       </c>
@@ -5202,7 +5203,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="51" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:32" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="25" t="s">
         <v>125</v>
       </c>
@@ -5225,7 +5226,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="102" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:32" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="s">
         <v>128</v>
       </c>
@@ -5274,10 +5275,10 @@
         <v>83</v>
       </c>
       <c r="S15" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="16" spans="1:32" ht="68" x14ac:dyDescent="0.2">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="16" spans="1:32" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
         <v>134</v>
       </c>
@@ -5349,10 +5350,10 @@
         <v>804</v>
       </c>
       <c r="S18" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
         <v>144</v>
       </c>
@@ -5375,7 +5376,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
         <v>149</v>
       </c>
@@ -5398,7 +5399,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
         <v>152</v>
       </c>
@@ -5421,7 +5422,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
         <v>155</v>
       </c>
@@ -5444,7 +5445,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="25" t="s">
         <v>158</v>
       </c>
@@ -5493,10 +5494,10 @@
         <v>84</v>
       </c>
       <c r="S24" s="27" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
         <v>164</v>
       </c>
@@ -5519,7 +5520,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="25" t="s">
         <v>166</v>
       </c>
@@ -5542,7 +5543,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:19" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="25" t="s">
         <v>168</v>
       </c>
@@ -5565,7 +5566,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="25" t="s">
         <v>171</v>
       </c>
@@ -5588,7 +5589,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="25" t="s">
         <v>174</v>
       </c>
@@ -5611,7 +5612,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="25" t="s">
         <v>177</v>
       </c>
@@ -5634,7 +5635,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="25" t="s">
         <v>180</v>
       </c>
@@ -5657,7 +5658,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="25" t="s">
         <v>183</v>
       </c>
@@ -5680,7 +5681,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="25" t="s">
         <v>186</v>
       </c>
@@ -5729,10 +5730,10 @@
         <v>85</v>
       </c>
       <c r="S34" s="27" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="s">
         <v>193</v>
       </c>
@@ -5755,7 +5756,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="25" t="s">
         <v>196</v>
       </c>
@@ -5778,7 +5779,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="25" t="s">
         <v>199</v>
       </c>
@@ -5801,7 +5802,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="25" t="s">
         <v>202</v>
       </c>
@@ -5824,7 +5825,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="25" t="s">
         <v>205</v>
       </c>
@@ -5847,7 +5848,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="25" t="s">
         <v>208</v>
       </c>
@@ -5870,7 +5871,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="25" t="s">
         <v>211</v>
       </c>
@@ -5962,7 +5963,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="25" t="s">
         <v>223</v>
       </c>
@@ -5985,7 +5986,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="25" t="s">
         <v>226</v>
       </c>
@@ -6031,7 +6032,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="25" t="s">
         <v>232</v>
       </c>
@@ -6103,10 +6104,10 @@
         <v>86</v>
       </c>
       <c r="S50" s="27" t="s">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="25" t="s">
         <v>241</v>
       </c>
@@ -6152,7 +6153,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="25" t="s">
         <v>246</v>
       </c>
@@ -6198,7 +6199,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="25" t="s">
         <v>252</v>
       </c>
@@ -6221,7 +6222,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="25" t="s">
         <v>255</v>
       </c>
@@ -6244,7 +6245,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="25" t="s">
         <v>258</v>
       </c>
@@ -6267,7 +6268,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="25" t="s">
         <v>261</v>
       </c>
@@ -6290,7 +6291,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="25" t="s">
         <v>264</v>
       </c>
@@ -6339,10 +6340,10 @@
         <v>800</v>
       </c>
       <c r="S60" s="27" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="61" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="61" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="25" t="s">
         <v>270</v>
       </c>
@@ -6365,7 +6366,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="25" t="s">
         <v>273</v>
       </c>
@@ -6388,7 +6389,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="25" t="s">
         <v>276</v>
       </c>
@@ -6411,7 +6412,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="25" t="s">
         <v>279</v>
       </c>
@@ -6434,7 +6435,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="25" t="s">
         <v>282</v>
       </c>
@@ -6457,7 +6458,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="25" t="s">
         <v>286</v>
       </c>
@@ -6480,7 +6481,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="25" t="s">
         <v>289</v>
       </c>
@@ -6503,7 +6504,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="25" t="s">
         <v>292</v>
       </c>
@@ -6526,7 +6527,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="25" t="s">
         <v>295</v>
       </c>
@@ -6549,7 +6550,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="70" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:19" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="25" t="s">
         <v>298</v>
       </c>
@@ -6572,7 +6573,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="25" t="s">
         <v>301</v>
       </c>
@@ -6595,7 +6596,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="72" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:19" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="25" t="s">
         <v>304</v>
       </c>
@@ -6618,7 +6619,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="73" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="25" t="s">
         <v>307</v>
       </c>
@@ -6687,13 +6688,13 @@
         <v>96</v>
       </c>
       <c r="R75" s="27" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="S75" s="27" t="s">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="76" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="76" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="25" t="s">
         <v>316</v>
       </c>
@@ -6739,7 +6740,7 @@
         <v>96</v>
       </c>
       <c r="R77" s="27" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="S77" s="27" t="s">
         <v>67</v>
@@ -6791,7 +6792,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="s">
         <v>328</v>
       </c>
@@ -6814,7 +6815,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" s="25" t="s">
         <v>331</v>
       </c>
@@ -6837,7 +6838,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" s="25" t="s">
         <v>334</v>
       </c>
@@ -6860,7 +6861,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" s="25" t="s">
         <v>337</v>
       </c>
@@ -6883,7 +6884,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="25" t="s">
         <v>340</v>
       </c>
@@ -6929,7 +6930,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="86" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="25" t="s">
         <v>346</v>
       </c>
@@ -6975,7 +6976,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" s="25" t="s">
         <v>352</v>
       </c>
@@ -6998,7 +6999,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="89" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="25" t="s">
         <v>355</v>
       </c>
@@ -7044,7 +7045,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="91" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="25" t="s">
         <v>360</v>
       </c>
@@ -7090,10 +7091,10 @@
         <v>92</v>
       </c>
       <c r="R92" s="27" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="S92" s="27" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="93" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -7104,7 +7105,7 @@
         <v>362</v>
       </c>
       <c r="C93" s="25" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="D93" s="25" t="s">
         <v>27</v>
@@ -7119,10 +7120,10 @@
         <v>92</v>
       </c>
       <c r="R93" s="27" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="S93" s="27" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="94" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -7148,7 +7149,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="95" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="25" t="s">
         <v>367</v>
       </c>
@@ -7171,7 +7172,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="96" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="25" t="s">
         <v>370</v>
       </c>
@@ -7194,7 +7195,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="97" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" s="25" t="s">
         <v>373</v>
       </c>
@@ -7263,7 +7264,7 @@
         <v>92</v>
       </c>
       <c r="R99" s="27" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="S99" s="27" t="s">
         <v>67</v>
@@ -7292,13 +7293,13 @@
         <v>92</v>
       </c>
       <c r="R100" s="27" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="S100" s="27" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="s">
         <v>384</v>
       </c>
@@ -7344,7 +7345,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="103" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:19" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="s">
         <v>389</v>
       </c>
@@ -7367,7 +7368,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="s">
         <v>392</v>
       </c>
@@ -7390,7 +7391,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="105" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="25" t="s">
         <v>395</v>
       </c>
@@ -7459,7 +7460,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="108" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="s">
         <v>404</v>
       </c>
@@ -7482,7 +7483,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="109" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" s="25" t="s">
         <v>407</v>
       </c>
@@ -7505,7 +7506,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="110" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="25" t="s">
         <v>410</v>
       </c>
@@ -7528,7 +7529,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="111" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="25" t="s">
         <v>413</v>
       </c>
@@ -7551,7 +7552,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="112" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" s="25" t="s">
         <v>416</v>
       </c>
@@ -7574,7 +7575,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="113" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" s="25" t="s">
         <v>418</v>
       </c>
@@ -7597,7 +7598,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="114" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="25" t="s">
         <v>421</v>
       </c>
@@ -7620,7 +7621,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="115" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" s="25" t="s">
         <v>424</v>
       </c>
@@ -7643,7 +7644,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="116" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" s="25" t="s">
         <v>427</v>
       </c>
@@ -7666,7 +7667,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="117" spans="1:16" ht="102" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:16" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" s="25" t="s">
         <v>430</v>
       </c>
@@ -7689,7 +7690,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="118" spans="1:16" ht="153" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:16" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="25" t="s">
         <v>433</v>
       </c>
@@ -7758,7 +7759,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="121" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="25" t="s">
         <v>442</v>
       </c>
@@ -7781,7 +7782,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="122" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:16" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="25" t="s">
         <v>445</v>
       </c>
@@ -7827,7 +7828,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="124" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="25" t="s">
         <v>451</v>
       </c>
@@ -7896,7 +7897,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="127" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" s="25" t="s">
         <v>461</v>
       </c>
@@ -7942,7 +7943,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="129" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" s="25" t="s">
         <v>467</v>
       </c>
@@ -7988,7 +7989,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="131" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="25" t="s">
         <v>473</v>
       </c>
@@ -8034,7 +8035,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="133" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="25" t="s">
         <v>479</v>
       </c>
@@ -8080,7 +8081,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="135" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="25" t="s">
         <v>485</v>
       </c>
@@ -8126,7 +8127,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="137" spans="1:16" ht="51" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:16" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="25" t="s">
         <v>491</v>
       </c>
@@ -8195,7 +8196,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="140" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="25" t="s">
         <v>500</v>
       </c>
@@ -8241,7 +8242,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="142" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="25" t="s">
         <v>506</v>
       </c>
@@ -8264,7 +8265,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="143" spans="1:16" ht="85" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:16" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="25" t="s">
         <v>509</v>
       </c>
@@ -8287,7 +8288,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="144" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" s="25" t="s">
         <v>512</v>
       </c>
@@ -8310,7 +8311,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="145" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="25" t="s">
         <v>515</v>
       </c>
@@ -8356,10 +8357,10 @@
         <v>92</v>
       </c>
       <c r="R146" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S146" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="147" spans="1:19" ht="170" x14ac:dyDescent="0.2">
@@ -8385,7 +8386,7 @@
         <v>92</v>
       </c>
       <c r="S147" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="148" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8411,10 +8412,10 @@
         <v>92</v>
       </c>
       <c r="R148" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S148" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="149" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8440,10 +8441,10 @@
         <v>92</v>
       </c>
       <c r="R149" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S149" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="150" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8469,10 +8470,10 @@
         <v>92</v>
       </c>
       <c r="R150" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S150" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="151" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8498,10 +8499,10 @@
         <v>92</v>
       </c>
       <c r="R151" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S151" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="152" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -8527,10 +8528,10 @@
         <v>92</v>
       </c>
       <c r="R152" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S152" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="153" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8556,10 +8557,10 @@
         <v>92</v>
       </c>
       <c r="R153" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S153" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="154" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8585,10 +8586,10 @@
         <v>92</v>
       </c>
       <c r="R154" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S154" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="155" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8614,10 +8615,10 @@
         <v>92</v>
       </c>
       <c r="R155" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S155" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="156" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8643,10 +8644,10 @@
         <v>92</v>
       </c>
       <c r="R156" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S156" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="157" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -8672,10 +8673,10 @@
         <v>92</v>
       </c>
       <c r="R157" s="27" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="S157" s="27" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="158" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -8704,10 +8705,10 @@
         <v>87</v>
       </c>
       <c r="S158" s="27" t="s">
-        <v>831</v>
-      </c>
-    </row>
-    <row r="159" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="159" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" s="25" t="s">
         <v>550</v>
       </c>
@@ -8730,7 +8731,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="160" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" s="25" t="s">
         <v>553</v>
       </c>
@@ -8753,7 +8754,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="161" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" s="25" t="s">
         <v>556</v>
       </c>
@@ -8776,7 +8777,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="162" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" s="25" t="s">
         <v>559</v>
       </c>
@@ -8799,7 +8800,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="163" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" s="25" t="s">
         <v>562</v>
       </c>
@@ -8822,7 +8823,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="164" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:19" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" s="25" t="s">
         <v>565</v>
       </c>
@@ -8845,7 +8846,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="165" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" s="25" t="s">
         <v>568</v>
       </c>
@@ -8868,7 +8869,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="166" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" s="25" t="s">
         <v>571</v>
       </c>
@@ -8891,7 +8892,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="167" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" s="25" t="s">
         <v>574</v>
       </c>
@@ -8914,7 +8915,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="168" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" s="25" t="s">
         <v>577</v>
       </c>
@@ -8937,7 +8938,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="169" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" s="25" t="s">
         <v>580</v>
       </c>
@@ -8960,7 +8961,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="170" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" s="25" t="s">
         <v>583</v>
       </c>
@@ -8983,7 +8984,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="171" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" s="25" t="s">
         <v>586</v>
       </c>
@@ -9006,7 +9007,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="172" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" s="25" t="s">
         <v>589</v>
       </c>
@@ -9029,7 +9030,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="173" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A173" s="25" t="s">
         <v>592</v>
       </c>
@@ -9075,13 +9076,13 @@
         <v>92</v>
       </c>
       <c r="R174" s="27" t="s">
-        <v>811</v>
+        <v>833</v>
       </c>
       <c r="S174" s="27" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="175" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="175" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" s="25" t="s">
         <v>598</v>
       </c>
@@ -9104,7 +9105,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="176" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" s="25" t="s">
         <v>601</v>
       </c>
@@ -9127,7 +9128,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="177" spans="1:22" ht="51" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:22" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" s="25" t="s">
         <v>604</v>
       </c>
@@ -9150,7 +9151,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="178" spans="1:22" ht="34" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:22" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" s="25" t="s">
         <v>607</v>
       </c>
@@ -9173,7 +9174,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="179" spans="1:22" ht="17" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:22" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" s="25" t="s">
         <v>610</v>
       </c>
@@ -9196,7 +9197,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="180" spans="1:22" ht="51" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:22" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" s="25" t="s">
         <v>613</v>
       </c>
@@ -9219,7 +9220,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="181" spans="1:22" ht="68" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:22" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" s="25" t="s">
         <v>616</v>
       </c>
@@ -9242,7 +9243,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="182" spans="1:22" ht="85" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:22" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" s="25" t="s">
         <v>619</v>
       </c>
@@ -9265,7 +9266,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="183" spans="1:22" ht="102" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:22" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" s="25" t="s">
         <v>622</v>
       </c>
@@ -9288,7 +9289,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="184" spans="1:22" ht="68" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:22" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" s="25" t="s">
         <v>625</v>
       </c>
@@ -9311,7 +9312,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="185" spans="1:22" ht="34" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:22" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" s="25" t="s">
         <v>628</v>
       </c>
@@ -9334,7 +9335,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="186" spans="1:22" ht="51" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:22" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" s="25" t="s">
         <v>631</v>
       </c>
@@ -9357,7 +9358,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="187" spans="1:22" ht="34" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:22" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" s="25" t="s">
         <v>634</v>
       </c>
@@ -9381,7 +9382,7 @@
       </c>
       <c r="V187" s="31"/>
     </row>
-    <row r="188" spans="1:22" ht="51" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:22" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" s="25" t="s">
         <v>637</v>
       </c>
@@ -9404,7 +9405,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="189" spans="1:22" ht="85" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:22" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" s="25" t="s">
         <v>640</v>
       </c>
@@ -9427,7 +9428,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="190" spans="1:22" ht="51" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:22" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" s="25" t="s">
         <v>643</v>
       </c>
@@ -9473,7 +9474,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="192" spans="1:22" ht="68" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:22" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" s="25" t="s">
         <v>649</v>
       </c>
@@ -9496,7 +9497,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="193" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" s="25" t="s">
         <v>652</v>
       </c>
@@ -9519,7 +9520,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="194" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" s="25" t="s">
         <v>655</v>
       </c>
@@ -9542,7 +9543,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="195" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" s="25" t="s">
         <v>658</v>
       </c>
@@ -9565,7 +9566,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="196" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A196" s="25" t="s">
         <v>661</v>
       </c>
@@ -9588,7 +9589,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="197" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" s="25" t="s">
         <v>664</v>
       </c>
@@ -9611,7 +9612,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="198" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" s="25" t="s">
         <v>667</v>
       </c>
@@ -9634,7 +9635,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="199" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" s="25" t="s">
         <v>670</v>
       </c>
@@ -9680,7 +9681,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="201" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A201" s="25" t="s">
         <v>676</v>
       </c>
@@ -9703,7 +9704,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="202" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" s="25" t="s">
         <v>679</v>
       </c>
@@ -9726,7 +9727,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="203" spans="1:19" ht="170" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:19" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" s="25" t="s">
         <v>682</v>
       </c>
@@ -9749,7 +9750,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="204" spans="1:19" ht="102" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:19" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A204" s="25" t="s">
         <v>685</v>
       </c>
@@ -9772,7 +9773,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="205" spans="1:19" ht="170" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:19" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A205" s="25" t="s">
         <v>688</v>
       </c>
@@ -9821,10 +9822,10 @@
         <v>810</v>
       </c>
       <c r="S206" s="27" t="s">
-        <v>829</v>
-      </c>
-    </row>
-    <row r="207" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="207" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A207" s="25" t="s">
         <v>695</v>
       </c>
@@ -9899,10 +9900,10 @@
         <v>89</v>
       </c>
       <c r="S209" s="27" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="210" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="210" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" s="25" t="s">
         <v>704</v>
       </c>
@@ -9925,7 +9926,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="211" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" s="25" t="s">
         <v>707</v>
       </c>
@@ -9948,7 +9949,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="212" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" s="25" t="s">
         <v>710</v>
       </c>
@@ -9971,7 +9972,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="213" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" s="25" t="s">
         <v>713</v>
       </c>
@@ -9994,7 +9995,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="214" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" s="25" t="s">
         <v>716</v>
       </c>
@@ -10017,7 +10018,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="215" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" s="25" t="s">
         <v>719</v>
       </c>
@@ -10040,7 +10041,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="216" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" s="25" t="s">
         <v>721</v>
       </c>
@@ -10063,7 +10064,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="217" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" s="25" t="s">
         <v>724</v>
       </c>
@@ -10086,7 +10087,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="218" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A218" s="25" t="s">
         <v>726</v>
       </c>
@@ -10109,7 +10110,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="219" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A219" s="25" t="s">
         <v>729</v>
       </c>
@@ -10132,7 +10133,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="220" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" s="25" t="s">
         <v>732</v>
       </c>
@@ -10178,7 +10179,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="222" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" s="25" t="s">
         <v>738</v>
       </c>
@@ -10201,7 +10202,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="223" spans="1:19" ht="136" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:19" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" s="25" t="s">
         <v>740</v>
       </c>
@@ -10224,7 +10225,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="224" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" s="25" t="s">
         <v>743</v>
       </c>
@@ -10247,7 +10248,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="225" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" s="25" t="s">
         <v>746</v>
       </c>
@@ -10270,7 +10271,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="226" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" s="25" t="s">
         <v>749</v>
       </c>
@@ -10316,7 +10317,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="228" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" s="25" t="s">
         <v>755</v>
       </c>
@@ -10339,7 +10340,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="229" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" s="25" t="s">
         <v>758</v>
       </c>
@@ -10362,7 +10363,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="230" spans="1:19" ht="119" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:19" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" s="25" t="s">
         <v>761</v>
       </c>
@@ -10385,7 +10386,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="231" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" s="25" t="s">
         <v>764</v>
       </c>
@@ -10408,7 +10409,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="232" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:19" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A232" s="25" t="s">
         <v>767</v>
       </c>
@@ -10480,10 +10481,10 @@
         <v>809</v>
       </c>
       <c r="S234" s="27" t="s">
-        <v>833</v>
-      </c>
-    </row>
-    <row r="235" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="235" spans="1:19" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" s="25" t="s">
         <v>775</v>
       </c>
@@ -10529,7 +10530,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="237" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" s="25" t="s">
         <v>781</v>
       </c>
@@ -10552,7 +10553,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="238" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:19" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A238" s="25" t="s">
         <v>784</v>
       </c>
@@ -10598,7 +10599,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="240" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" s="25" t="s">
         <v>790</v>
       </c>
@@ -10621,7 +10622,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="241" spans="1:16" ht="68" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:16" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" s="25" t="s">
         <v>793</v>
       </c>
@@ -10644,259 +10645,259 @@
         <v>96</v>
       </c>
     </row>
-    <row r="242" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B242" s="32"/>
     </row>
-    <row r="243" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B243" s="32"/>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B244" s="32"/>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B245" s="32"/>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B246" s="32"/>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B247" s="32"/>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B248" s="32"/>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B249" s="32"/>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B250" s="32"/>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B251" s="32"/>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B252" s="32"/>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B253" s="32"/>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B254" s="32"/>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B255" s="32"/>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B256" s="32"/>
     </row>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="257" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B257" s="32"/>
     </row>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="258" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B258" s="32"/>
     </row>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="259" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B259" s="32"/>
     </row>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="260" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B260" s="32"/>
     </row>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="261" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B261" s="32"/>
     </row>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="262" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B262" s="32"/>
     </row>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="263" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B263" s="32"/>
     </row>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="264" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B264" s="32"/>
     </row>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="265" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B265" s="32"/>
     </row>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="266" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B266" s="32"/>
     </row>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="267" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B267" s="32"/>
     </row>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="268" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B268" s="32"/>
     </row>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="269" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B269" s="32"/>
     </row>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="270" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B270" s="32"/>
     </row>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="271" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B271" s="32"/>
     </row>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="272" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B272" s="32"/>
     </row>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="273" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B273" s="32"/>
     </row>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="274" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B274" s="32"/>
     </row>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="275" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B275" s="32"/>
     </row>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="276" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B276" s="32"/>
     </row>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="277" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B277" s="32"/>
     </row>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="278" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B278" s="32"/>
     </row>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="279" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B279" s="32"/>
     </row>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="280" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B280" s="32"/>
     </row>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="281" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B281" s="32"/>
     </row>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="282" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B282" s="32"/>
     </row>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="283" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B283" s="32"/>
     </row>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="284" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B284" s="32"/>
     </row>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="285" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B285" s="32"/>
     </row>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="286" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B286" s="32"/>
     </row>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="287" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B287" s="32"/>
     </row>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="288" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B288" s="32"/>
     </row>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="289" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B289" s="32"/>
     </row>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="290" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B290" s="32"/>
     </row>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="291" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B291" s="32"/>
     </row>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="292" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B292" s="32"/>
     </row>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="293" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B293" s="32"/>
     </row>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="294" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B294" s="32"/>
     </row>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="295" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B295" s="32"/>
     </row>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="296" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B296" s="32"/>
     </row>
-    <row r="297" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="297" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B297" s="32"/>
     </row>
-    <row r="298" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="298" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B298" s="32"/>
     </row>
-    <row r="299" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="299" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B299" s="32"/>
     </row>
-    <row r="300" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="300" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B300" s="32"/>
     </row>
-    <row r="301" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="301" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B301" s="32"/>
     </row>
-    <row r="302" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="302" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B302" s="32"/>
     </row>
-    <row r="303" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="303" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B303" s="32"/>
     </row>
-    <row r="304" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="304" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B304" s="32"/>
     </row>
-    <row r="305" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="305" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B305" s="32"/>
     </row>
-    <row r="306" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="306" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B306" s="32"/>
     </row>
-    <row r="307" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="307" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B307" s="32"/>
     </row>
-    <row r="308" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="308" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B308" s="32"/>
     </row>
-    <row r="309" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="309" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B309" s="32"/>
     </row>
-    <row r="310" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="310" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B310" s="32"/>
     </row>
-    <row r="311" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="311" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B311" s="32"/>
     </row>
-    <row r="312" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="312" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B312" s="32"/>
     </row>
-    <row r="313" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="313" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B313" s="32"/>
     </row>
-    <row r="314" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="314" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B314" s="32"/>
     </row>
-    <row r="315" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="315" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B315" s="32"/>
     </row>
-    <row r="316" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="316" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B316" s="32"/>
     </row>
-    <row r="317" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="317" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B317" s="32"/>
     </row>
-    <row r="318" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="318" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B318" s="32"/>
     </row>
-    <row r="319" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="319" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B319" s="32"/>
     </row>
-    <row r="320" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="320" spans="2:2" hidden="1" x14ac:dyDescent="0.2">
       <c r="B320" s="32"/>
     </row>
-    <row r="321" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="321" spans="2:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="B321" s="32"/>
     </row>
-    <row r="322" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="322" spans="2:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="B322" s="32"/>
     </row>
-    <row r="323" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="323" spans="2:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="B323" s="32"/>
     </row>
-    <row r="324" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="324" spans="2:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="B324" s="32"/>
     </row>
-    <row r="325" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="325" spans="2:14" hidden="1" x14ac:dyDescent="0.2">
       <c r="B325" s="32"/>
     </row>
-    <row r="326" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="326" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M326" s="30" t="str" cm="1">
         <f t="array" ref="M326">PAGE_NAME(B326)</f>
         <v/>
@@ -10906,7 +10907,7 @@
         <v/>
       </c>
     </row>
-    <row r="327" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="327" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M327" s="30" t="str" cm="1">
         <f t="array" ref="M327">PAGE_NAME(B327)</f>
         <v/>
@@ -10916,7 +10917,7 @@
         <v/>
       </c>
     </row>
-    <row r="328" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="328" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M328" s="30" t="str" cm="1">
         <f t="array" ref="M328">PAGE_NAME(B328)</f>
         <v/>
@@ -10926,7 +10927,7 @@
         <v/>
       </c>
     </row>
-    <row r="329" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="329" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M329" s="30" t="str" cm="1">
         <f t="array" ref="M329">PAGE_NAME(B329)</f>
         <v/>
@@ -10936,7 +10937,7 @@
         <v/>
       </c>
     </row>
-    <row r="330" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="330" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M330" s="30" t="str" cm="1">
         <f t="array" ref="M330">PAGE_NAME(B330)</f>
         <v/>
@@ -10946,7 +10947,7 @@
         <v/>
       </c>
     </row>
-    <row r="331" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="331" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M331" s="30" t="str" cm="1">
         <f t="array" ref="M331">PAGE_NAME(B331)</f>
         <v/>
@@ -10956,7 +10957,7 @@
         <v/>
       </c>
     </row>
-    <row r="332" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="332" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M332" s="30" t="str" cm="1">
         <f t="array" ref="M332">PAGE_NAME(B332)</f>
         <v/>
@@ -10966,7 +10967,7 @@
         <v/>
       </c>
     </row>
-    <row r="333" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="333" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M333" s="30" t="str" cm="1">
         <f t="array" ref="M333">PAGE_NAME(B333)</f>
         <v/>
@@ -10976,7 +10977,7 @@
         <v/>
       </c>
     </row>
-    <row r="334" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="334" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M334" s="30" t="str" cm="1">
         <f t="array" ref="M334">PAGE_NAME(B334)</f>
         <v/>
@@ -10986,7 +10987,7 @@
         <v/>
       </c>
     </row>
-    <row r="335" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="335" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M335" s="30" t="str" cm="1">
         <f t="array" ref="M335">PAGE_NAME(B335)</f>
         <v/>
@@ -10996,7 +10997,7 @@
         <v/>
       </c>
     </row>
-    <row r="336" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="336" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M336" s="30" t="str" cm="1">
         <f t="array" ref="M336">PAGE_NAME(B336)</f>
         <v/>
@@ -11006,7 +11007,7 @@
         <v/>
       </c>
     </row>
-    <row r="337" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="337" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M337" s="30" t="str" cm="1">
         <f t="array" ref="M337">PAGE_NAME(B337)</f>
         <v/>
@@ -11016,7 +11017,7 @@
         <v/>
       </c>
     </row>
-    <row r="338" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="338" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M338" s="30" t="str" cm="1">
         <f t="array" ref="M338">PAGE_NAME(B338)</f>
         <v/>
@@ -11026,7 +11027,7 @@
         <v/>
       </c>
     </row>
-    <row r="339" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="339" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M339" s="30" t="str" cm="1">
         <f t="array" ref="M339">PAGE_NAME(B339)</f>
         <v/>
@@ -11036,7 +11037,7 @@
         <v/>
       </c>
     </row>
-    <row r="340" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="340" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M340" s="30" t="str" cm="1">
         <f t="array" ref="M340">PAGE_NAME(B340)</f>
         <v/>
@@ -11046,7 +11047,7 @@
         <v/>
       </c>
     </row>
-    <row r="341" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="341" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M341" s="30" t="str" cm="1">
         <f t="array" ref="M341">PAGE_NAME(B341)</f>
         <v/>
@@ -11056,7 +11057,7 @@
         <v/>
       </c>
     </row>
-    <row r="342" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="342" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M342" s="30" t="str" cm="1">
         <f t="array" ref="M342">PAGE_NAME(B342)</f>
         <v/>
@@ -11066,7 +11067,7 @@
         <v/>
       </c>
     </row>
-    <row r="343" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="343" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M343" s="30" t="str" cm="1">
         <f t="array" ref="M343">PAGE_NAME(B343)</f>
         <v/>
@@ -11076,7 +11077,7 @@
         <v/>
       </c>
     </row>
-    <row r="344" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="344" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M344" s="30" t="str" cm="1">
         <f t="array" ref="M344">PAGE_NAME(B344)</f>
         <v/>
@@ -11086,7 +11087,7 @@
         <v/>
       </c>
     </row>
-    <row r="345" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="345" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M345" s="30" t="str" cm="1">
         <f t="array" ref="M345">PAGE_NAME(B345)</f>
         <v/>
@@ -11096,7 +11097,7 @@
         <v/>
       </c>
     </row>
-    <row r="346" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="346" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="B346" s="32"/>
       <c r="M346" s="30" t="str" cm="1">
         <f t="array" ref="M346">PAGE_NAME(B346)</f>
@@ -11107,7 +11108,7 @@
         <v/>
       </c>
     </row>
-    <row r="347" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="347" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M347" s="30" t="str" cm="1">
         <f t="array" ref="M347">PAGE_NAME(B347)</f>
         <v/>
@@ -11117,7 +11118,7 @@
         <v/>
       </c>
     </row>
-    <row r="348" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="348" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M348" s="30" t="str" cm="1">
         <f t="array" ref="M348">PAGE_NAME(B348)</f>
         <v/>
@@ -11127,7 +11128,7 @@
         <v/>
       </c>
     </row>
-    <row r="349" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="349" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M349" s="30" t="str" cm="1">
         <f t="array" ref="M349">PAGE_NAME(B349)</f>
         <v/>
@@ -11137,7 +11138,7 @@
         <v/>
       </c>
     </row>
-    <row r="350" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="350" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M350" s="30" t="str" cm="1">
         <f t="array" ref="M350">PAGE_NAME(B350)</f>
         <v/>
@@ -11147,7 +11148,7 @@
         <v/>
       </c>
     </row>
-    <row r="351" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="351" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M351" s="30" t="str" cm="1">
         <f t="array" ref="M351">PAGE_NAME(B351)</f>
         <v/>
@@ -11157,7 +11158,7 @@
         <v/>
       </c>
     </row>
-    <row r="352" spans="2:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="352" spans="2:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M352" s="30" t="str" cm="1">
         <f t="array" ref="M352">PAGE_NAME(B352)</f>
         <v/>
@@ -11167,7 +11168,7 @@
         <v/>
       </c>
     </row>
-    <row r="353" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="353" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M353" s="30" t="str" cm="1">
         <f t="array" ref="M353">PAGE_NAME(B353)</f>
         <v/>
@@ -11177,7 +11178,7 @@
         <v/>
       </c>
     </row>
-    <row r="354" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="354" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M354" s="30" t="str" cm="1">
         <f t="array" ref="M354">PAGE_NAME(B354)</f>
         <v/>
@@ -11187,7 +11188,7 @@
         <v/>
       </c>
     </row>
-    <row r="355" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="355" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M355" s="30" t="str" cm="1">
         <f t="array" ref="M355">PAGE_NAME(B355)</f>
         <v/>
@@ -11197,7 +11198,7 @@
         <v/>
       </c>
     </row>
-    <row r="356" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="356" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M356" s="30" t="str" cm="1">
         <f t="array" ref="M356">PAGE_NAME(B356)</f>
         <v/>
@@ -11207,7 +11208,7 @@
         <v/>
       </c>
     </row>
-    <row r="357" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="357" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M357" s="30" t="str" cm="1">
         <f t="array" ref="M357">PAGE_NAME(B357)</f>
         <v/>
@@ -11217,7 +11218,7 @@
         <v/>
       </c>
     </row>
-    <row r="358" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="358" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M358" s="30" t="str" cm="1">
         <f t="array" ref="M358">PAGE_NAME(B358)</f>
         <v/>
@@ -11227,7 +11228,7 @@
         <v/>
       </c>
     </row>
-    <row r="359" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="359" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M359" s="30" t="str" cm="1">
         <f t="array" ref="M359">PAGE_NAME(B359)</f>
         <v/>
@@ -11237,7 +11238,7 @@
         <v/>
       </c>
     </row>
-    <row r="360" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="360" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M360" s="30" t="str" cm="1">
         <f t="array" ref="M360">PAGE_NAME(B360)</f>
         <v/>
@@ -11247,7 +11248,7 @@
         <v/>
       </c>
     </row>
-    <row r="361" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="361" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M361" s="30" t="str" cm="1">
         <f t="array" ref="M361">PAGE_NAME(B361)</f>
         <v/>
@@ -11257,7 +11258,7 @@
         <v/>
       </c>
     </row>
-    <row r="362" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="362" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M362" s="30" t="str" cm="1">
         <f t="array" ref="M362">PAGE_NAME(B362)</f>
         <v/>
@@ -11267,7 +11268,7 @@
         <v/>
       </c>
     </row>
-    <row r="363" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="363" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M363" s="30" t="str" cm="1">
         <f t="array" ref="M363">PAGE_NAME(B363)</f>
         <v/>
@@ -11277,7 +11278,7 @@
         <v/>
       </c>
     </row>
-    <row r="364" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="364" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M364" s="30" t="str" cm="1">
         <f t="array" ref="M364">PAGE_NAME(B364)</f>
         <v/>
@@ -11287,7 +11288,7 @@
         <v/>
       </c>
     </row>
-    <row r="365" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="365" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M365" s="30" t="str" cm="1">
         <f t="array" ref="M365">PAGE_NAME(B365)</f>
         <v/>
@@ -11297,7 +11298,7 @@
         <v/>
       </c>
     </row>
-    <row r="366" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="366" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M366" s="30" t="str" cm="1">
         <f t="array" ref="M366">PAGE_NAME(B366)</f>
         <v/>
@@ -11307,7 +11308,7 @@
         <v/>
       </c>
     </row>
-    <row r="367" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="367" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M367" s="30" t="str" cm="1">
         <f t="array" ref="M367">PAGE_NAME(B367)</f>
         <v/>
@@ -11317,7 +11318,7 @@
         <v/>
       </c>
     </row>
-    <row r="368" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="368" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M368" s="30" t="str" cm="1">
         <f t="array" ref="M368">PAGE_NAME(B368)</f>
         <v/>
@@ -11327,7 +11328,7 @@
         <v/>
       </c>
     </row>
-    <row r="369" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="369" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M369" s="30" t="str" cm="1">
         <f t="array" ref="M369">PAGE_NAME(B369)</f>
         <v/>
@@ -11337,7 +11338,7 @@
         <v/>
       </c>
     </row>
-    <row r="370" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="370" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M370" s="30" t="str" cm="1">
         <f t="array" ref="M370">PAGE_NAME(B370)</f>
         <v/>
@@ -11347,7 +11348,7 @@
         <v/>
       </c>
     </row>
-    <row r="371" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="371" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M371" s="30" t="str" cm="1">
         <f t="array" ref="M371">PAGE_NAME(B371)</f>
         <v/>
@@ -11357,7 +11358,7 @@
         <v/>
       </c>
     </row>
-    <row r="372" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="372" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M372" s="30" t="str" cm="1">
         <f t="array" ref="M372">PAGE_NAME(B372)</f>
         <v/>
@@ -11367,7 +11368,7 @@
         <v/>
       </c>
     </row>
-    <row r="373" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="373" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M373" s="30" t="str" cm="1">
         <f t="array" ref="M373">PAGE_NAME(B373)</f>
         <v/>
@@ -11377,7 +11378,7 @@
         <v/>
       </c>
     </row>
-    <row r="374" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="374" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M374" s="30" t="str" cm="1">
         <f t="array" ref="M374">PAGE_NAME(B374)</f>
         <v/>
@@ -11387,7 +11388,7 @@
         <v/>
       </c>
     </row>
-    <row r="375" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="375" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M375" s="30" t="str" cm="1">
         <f t="array" ref="M375">PAGE_NAME(B375)</f>
         <v/>
@@ -11397,7 +11398,7 @@
         <v/>
       </c>
     </row>
-    <row r="376" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="376" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M376" s="30" t="str" cm="1">
         <f t="array" ref="M376">PAGE_NAME(B376)</f>
         <v/>
@@ -11407,7 +11408,7 @@
         <v/>
       </c>
     </row>
-    <row r="377" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="377" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M377" s="30" t="str" cm="1">
         <f t="array" ref="M377">PAGE_NAME(B377)</f>
         <v/>
@@ -11417,7 +11418,7 @@
         <v/>
       </c>
     </row>
-    <row r="378" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="378" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M378" s="30" t="str" cm="1">
         <f t="array" ref="M378">PAGE_NAME(B378)</f>
         <v/>
@@ -11427,7 +11428,7 @@
         <v/>
       </c>
     </row>
-    <row r="379" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="379" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M379" s="30" t="str" cm="1">
         <f t="array" ref="M379">PAGE_NAME(B379)</f>
         <v/>
@@ -11437,7 +11438,7 @@
         <v/>
       </c>
     </row>
-    <row r="380" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="380" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M380" s="30" t="str" cm="1">
         <f t="array" ref="M380">PAGE_NAME(B380)</f>
         <v/>
@@ -11447,7 +11448,7 @@
         <v/>
       </c>
     </row>
-    <row r="381" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="381" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M381" s="30" t="str" cm="1">
         <f t="array" ref="M381">PAGE_NAME(B381)</f>
         <v/>
@@ -11457,7 +11458,7 @@
         <v/>
       </c>
     </row>
-    <row r="382" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="382" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M382" s="30" t="str" cm="1">
         <f t="array" ref="M382">PAGE_NAME(B382)</f>
         <v/>
@@ -11467,7 +11468,7 @@
         <v/>
       </c>
     </row>
-    <row r="383" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="383" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M383" s="30" t="str" cm="1">
         <f t="array" ref="M383">PAGE_NAME(B383)</f>
         <v/>
@@ -11477,7 +11478,7 @@
         <v/>
       </c>
     </row>
-    <row r="384" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="384" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M384" s="30" t="str" cm="1">
         <f t="array" ref="M384">PAGE_NAME(B384)</f>
         <v/>
@@ -11487,7 +11488,7 @@
         <v/>
       </c>
     </row>
-    <row r="385" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="385" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M385" s="30" t="str" cm="1">
         <f t="array" ref="M385">PAGE_NAME(B385)</f>
         <v/>
@@ -11497,7 +11498,7 @@
         <v/>
       </c>
     </row>
-    <row r="386" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="386" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M386" s="30" t="str" cm="1">
         <f t="array" ref="M386">PAGE_NAME(B386)</f>
         <v/>
@@ -11507,7 +11508,7 @@
         <v/>
       </c>
     </row>
-    <row r="387" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="387" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M387" s="30" t="str" cm="1">
         <f t="array" ref="M387">PAGE_NAME(B387)</f>
         <v/>
@@ -11517,7 +11518,7 @@
         <v/>
       </c>
     </row>
-    <row r="388" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="388" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M388" s="30" t="str" cm="1">
         <f t="array" ref="M388">PAGE_NAME(B388)</f>
         <v/>
@@ -11527,7 +11528,7 @@
         <v/>
       </c>
     </row>
-    <row r="389" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="389" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M389" s="30" t="str" cm="1">
         <f t="array" ref="M389">PAGE_NAME(B389)</f>
         <v/>
@@ -11537,7 +11538,7 @@
         <v/>
       </c>
     </row>
-    <row r="390" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="390" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M390" s="30" t="str" cm="1">
         <f t="array" ref="M390">PAGE_NAME(B390)</f>
         <v/>
@@ -11547,7 +11548,7 @@
         <v/>
       </c>
     </row>
-    <row r="391" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="391" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M391" s="30" t="str" cm="1">
         <f t="array" ref="M391">PAGE_NAME(B391)</f>
         <v/>
@@ -11557,7 +11558,7 @@
         <v/>
       </c>
     </row>
-    <row r="392" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="392" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M392" s="30" t="str" cm="1">
         <f t="array" ref="M392">PAGE_NAME(B392)</f>
         <v/>
@@ -11567,7 +11568,7 @@
         <v/>
       </c>
     </row>
-    <row r="393" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="393" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M393" s="30" t="str" cm="1">
         <f t="array" ref="M393">PAGE_NAME(B393)</f>
         <v/>
@@ -11577,7 +11578,7 @@
         <v/>
       </c>
     </row>
-    <row r="394" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="394" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M394" s="30" t="str" cm="1">
         <f t="array" ref="M394">PAGE_NAME(B394)</f>
         <v/>
@@ -11587,7 +11588,7 @@
         <v/>
       </c>
     </row>
-    <row r="395" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="395" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M395" s="30" t="str" cm="1">
         <f t="array" ref="M395">PAGE_NAME(B395)</f>
         <v/>
@@ -11597,7 +11598,7 @@
         <v/>
       </c>
     </row>
-    <row r="396" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="396" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M396" s="30" t="str" cm="1">
         <f t="array" ref="M396">PAGE_NAME(B396)</f>
         <v/>
@@ -11607,7 +11608,7 @@
         <v/>
       </c>
     </row>
-    <row r="397" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="397" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M397" s="30" t="str" cm="1">
         <f t="array" ref="M397">PAGE_NAME(B397)</f>
         <v/>
@@ -11617,7 +11618,7 @@
         <v/>
       </c>
     </row>
-    <row r="398" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="398" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M398" s="30" t="str" cm="1">
         <f t="array" ref="M398">PAGE_NAME(B398)</f>
         <v/>
@@ -11627,7 +11628,7 @@
         <v/>
       </c>
     </row>
-    <row r="399" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="399" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M399" s="30" t="str" cm="1">
         <f t="array" ref="M399">PAGE_NAME(B399)</f>
         <v/>
@@ -11637,7 +11638,7 @@
         <v/>
       </c>
     </row>
-    <row r="400" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="400" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M400" s="30" t="str" cm="1">
         <f t="array" ref="M400">PAGE_NAME(B400)</f>
         <v/>
@@ -11647,7 +11648,7 @@
         <v/>
       </c>
     </row>
-    <row r="401" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="401" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M401" s="30" t="str" cm="1">
         <f t="array" ref="M401">PAGE_NAME(B401)</f>
         <v/>
@@ -11657,7 +11658,7 @@
         <v/>
       </c>
     </row>
-    <row r="402" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="402" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M402" s="30" t="str" cm="1">
         <f t="array" ref="M402">PAGE_NAME(B402)</f>
         <v/>
@@ -11667,7 +11668,7 @@
         <v/>
       </c>
     </row>
-    <row r="403" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="403" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M403" s="30" t="str" cm="1">
         <f t="array" ref="M403">PAGE_NAME(B403)</f>
         <v/>
@@ -11677,7 +11678,7 @@
         <v/>
       </c>
     </row>
-    <row r="404" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="404" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M404" s="30" t="str" cm="1">
         <f t="array" ref="M404">PAGE_NAME(B404)</f>
         <v/>
@@ -11687,7 +11688,7 @@
         <v/>
       </c>
     </row>
-    <row r="405" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="405" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M405" s="30" t="str" cm="1">
         <f t="array" ref="M405">PAGE_NAME(B405)</f>
         <v/>
@@ -11697,7 +11698,7 @@
         <v/>
       </c>
     </row>
-    <row r="406" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="406" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M406" s="30" t="str" cm="1">
         <f t="array" ref="M406">PAGE_NAME(B406)</f>
         <v/>
@@ -11707,7 +11708,7 @@
         <v/>
       </c>
     </row>
-    <row r="407" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="407" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M407" s="30" t="str" cm="1">
         <f t="array" ref="M407">PAGE_NAME(B407)</f>
         <v/>
@@ -11717,7 +11718,7 @@
         <v/>
       </c>
     </row>
-    <row r="408" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="408" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M408" s="30" t="str" cm="1">
         <f t="array" ref="M408">PAGE_NAME(B408)</f>
         <v/>
@@ -11727,7 +11728,7 @@
         <v/>
       </c>
     </row>
-    <row r="409" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="409" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M409" s="30" t="str" cm="1">
         <f t="array" ref="M409">PAGE_NAME(B409)</f>
         <v/>
@@ -11737,7 +11738,7 @@
         <v/>
       </c>
     </row>
-    <row r="410" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="410" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M410" s="30" t="str" cm="1">
         <f t="array" ref="M410">PAGE_NAME(B410)</f>
         <v/>
@@ -11747,7 +11748,7 @@
         <v/>
       </c>
     </row>
-    <row r="411" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="411" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M411" s="30" t="str" cm="1">
         <f t="array" ref="M411">PAGE_NAME(B411)</f>
         <v/>
@@ -11757,7 +11758,7 @@
         <v/>
       </c>
     </row>
-    <row r="412" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="412" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M412" s="30" t="str" cm="1">
         <f t="array" ref="M412">PAGE_NAME(B412)</f>
         <v/>
@@ -11767,7 +11768,7 @@
         <v/>
       </c>
     </row>
-    <row r="413" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="413" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M413" s="30" t="str" cm="1">
         <f t="array" ref="M413">PAGE_NAME(B413)</f>
         <v/>
@@ -11777,7 +11778,7 @@
         <v/>
       </c>
     </row>
-    <row r="414" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="414" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M414" s="30" t="str" cm="1">
         <f t="array" ref="M414">PAGE_NAME(B414)</f>
         <v/>
@@ -11787,7 +11788,7 @@
         <v/>
       </c>
     </row>
-    <row r="415" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="415" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M415" s="30" t="str" cm="1">
         <f t="array" ref="M415">PAGE_NAME(B415)</f>
         <v/>
@@ -11797,7 +11798,7 @@
         <v/>
       </c>
     </row>
-    <row r="416" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="416" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M416" s="30" t="str" cm="1">
         <f t="array" ref="M416">PAGE_NAME(B416)</f>
         <v/>
@@ -11807,7 +11808,7 @@
         <v/>
       </c>
     </row>
-    <row r="417" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="417" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M417" s="30" t="str" cm="1">
         <f t="array" ref="M417">PAGE_NAME(B417)</f>
         <v/>
@@ -11817,7 +11818,7 @@
         <v/>
       </c>
     </row>
-    <row r="418" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="418" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M418" s="30" t="str" cm="1">
         <f t="array" ref="M418">PAGE_NAME(B418)</f>
         <v/>
@@ -11827,7 +11828,7 @@
         <v/>
       </c>
     </row>
-    <row r="419" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="419" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M419" s="30" t="str" cm="1">
         <f t="array" ref="M419">PAGE_NAME(B419)</f>
         <v/>
@@ -11837,7 +11838,7 @@
         <v/>
       </c>
     </row>
-    <row r="420" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="420" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M420" s="30" t="str" cm="1">
         <f t="array" ref="M420">PAGE_NAME(B420)</f>
         <v/>
@@ -11847,7 +11848,7 @@
         <v/>
       </c>
     </row>
-    <row r="421" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="421" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M421" s="30" t="str" cm="1">
         <f t="array" ref="M421">PAGE_NAME(B421)</f>
         <v/>
@@ -11857,7 +11858,7 @@
         <v/>
       </c>
     </row>
-    <row r="422" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="422" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M422" s="30" t="str" cm="1">
         <f t="array" ref="M422">PAGE_NAME(B422)</f>
         <v/>
@@ -11867,7 +11868,7 @@
         <v/>
       </c>
     </row>
-    <row r="423" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="423" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M423" s="30" t="str" cm="1">
         <f t="array" ref="M423">PAGE_NAME(B423)</f>
         <v/>
@@ -11877,7 +11878,7 @@
         <v/>
       </c>
     </row>
-    <row r="424" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="424" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M424" s="30" t="str" cm="1">
         <f t="array" ref="M424">PAGE_NAME(B424)</f>
         <v/>
@@ -11887,7 +11888,7 @@
         <v/>
       </c>
     </row>
-    <row r="425" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="425" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M425" s="30" t="str" cm="1">
         <f t="array" ref="M425">PAGE_NAME(B425)</f>
         <v/>
@@ -11897,7 +11898,7 @@
         <v/>
       </c>
     </row>
-    <row r="426" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="426" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M426" s="30" t="str" cm="1">
         <f t="array" ref="M426">PAGE_NAME(B426)</f>
         <v/>
@@ -11907,7 +11908,7 @@
         <v/>
       </c>
     </row>
-    <row r="427" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="427" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M427" s="30" t="str" cm="1">
         <f t="array" ref="M427">PAGE_NAME(B427)</f>
         <v/>
@@ -11917,7 +11918,7 @@
         <v/>
       </c>
     </row>
-    <row r="428" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="428" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M428" s="30" t="str" cm="1">
         <f t="array" ref="M428">PAGE_NAME(B428)</f>
         <v/>
@@ -11927,7 +11928,7 @@
         <v/>
       </c>
     </row>
-    <row r="429" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="429" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M429" s="30" t="str" cm="1">
         <f t="array" ref="M429">PAGE_NAME(B429)</f>
         <v/>
@@ -11937,7 +11938,7 @@
         <v/>
       </c>
     </row>
-    <row r="430" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="430" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M430" s="30" t="str" cm="1">
         <f t="array" ref="M430">PAGE_NAME(B430)</f>
         <v/>
@@ -11947,7 +11948,7 @@
         <v/>
       </c>
     </row>
-    <row r="431" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="431" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M431" s="30" t="str" cm="1">
         <f t="array" ref="M431">PAGE_NAME(B431)</f>
         <v/>
@@ -11957,7 +11958,7 @@
         <v/>
       </c>
     </row>
-    <row r="432" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="432" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M432" s="30" t="str" cm="1">
         <f t="array" ref="M432">PAGE_NAME(B432)</f>
         <v/>
@@ -11967,7 +11968,7 @@
         <v/>
       </c>
     </row>
-    <row r="433" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="433" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M433" s="30" t="str" cm="1">
         <f t="array" ref="M433">PAGE_NAME(B433)</f>
         <v/>
@@ -11977,7 +11978,7 @@
         <v/>
       </c>
     </row>
-    <row r="434" spans="13:14" ht="17" x14ac:dyDescent="0.2">
+    <row r="434" spans="13:14" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="M434" s="30" t="str" cm="1">
         <f t="array" ref="M434">PAGE_NAME(B434)</f>
         <v/>
@@ -11988,10 +11989,24 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U434" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}"/>
+  <autoFilter ref="A1:U434" xr:uid="{0272D98A-080C-3945-A7E0-CB54FB3A65A9}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="SHALL"/>
+        <filter val="SHALL NOT"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="CRD Client"/>
+        <filter val="CRD Client, CRD Server"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="19" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B24" r:id="rId1" location="ci-c-dev-3" xr:uid="{09A37A58-2BBF-FA48-99E7-8234535ED081}"/>
+    <hyperlink ref="B92" r:id="rId2" location="ci-c-found-36" xr:uid="{E9061C6B-069C-4F41-865D-1DCDB9B7CD5D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>

</xml_diff>

<commit_message>
ID-130: request logical model validation fixes (#89)
* clean up request validation using logical models, including adding CRD profile checks

* Update client vs server presets to have passing requests

* update requirements mapping

* fixes found during testing
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219F36C1-5EB6-A945-A337-8475063D37E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C32B42-E0C4-1644-B729-71604343D353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="760" windowWidth="34240" windowHeight="21260" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1630" uniqueCount="840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="844">
   <si>
     <r>
       <rPr>
@@ -2955,18 +2955,12 @@
     <t>https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-no-order.html#ci-c-prof-1</t>
   </si>
   <si>
-    <t>CRD Clients **SHALL** use either this Appointment with Order profile and/or the [with-order](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-with-order.html) to provide `appointments` context objects to CRD Servers when invoking the [appointment-book](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/hooks.html#appointment-book) hook as well as to [resolve other references](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/foundation.html#additional-data-retrieval) to Appointment resources.</t>
-  </si>
-  <si>
     <t>prof-2</t>
   </si>
   <si>
     <t>https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-with-order.html#ci-c-prof-2</t>
   </si>
   <si>
-    <t>CRD Clients **SHALL** use either this Appointment without Order and/or the [no-order](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-no-order.html) to provide `appointments` context objects to CRD Servers when invoking the [appointment-book](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/hooks.html#appointment-book) hook as well as to [resolve other references](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/foundation.html#additional-data-retrieval) to Appointment resources.</t>
-  </si>
-  <si>
     <t>prof-3</t>
   </si>
   <si>
@@ -3894,9 +3888,6 @@
     <t>Limitation: future</t>
   </si>
   <si>
-    <t>ID-125</t>
-  </si>
-  <si>
     <t>Limitation: what-if not included at this time</t>
   </si>
   <si>
@@ -3910,6 +3901,27 @@
   </si>
   <si>
     <t>Limitation: SMART launch card details not verified at present</t>
+  </si>
+  <si>
+    <t>Mechanical: logical model</t>
+  </si>
+  <si>
+    <t>Mechanical: check for the coverage-information response type across all calls to this hook</t>
+  </si>
+  <si>
+    <t>Mechanical: Inferno checks only the external exchange</t>
+  </si>
+  <si>
+    <t>CRD Clients **SHALL** use either this Appointment without Order profile and/or the [with-order](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-with-order.html) to provide `appointments` context objects to CRD Servers when invoking the [appointment-book](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/hooks.html#appointment-book) hook as well as to [resolve other references](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/foundation.html#additional-data-retrieval) to Appointment resources.</t>
+  </si>
+  <si>
+    <t>CRD Clients **SHALL** use either this Appointment with Order and/or the [no-order](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/StructureDefinition-profile-appointment-no-order.html) to provide `appointments` context objects to CRD Servers when invoking the [appointment-book](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/hooks.html#appointment-book) hook as well as to [resolve other references](https://hl7.org/fhir/us/davinci-crd/2.2.1/en/foundation.html#additional-data-retrieval) to Appointment resources.</t>
+  </si>
+  <si>
+    <t>NOTE: corrected Appointment without Order -&gt; Appointement with Order</t>
+  </si>
+  <si>
+    <t>NOTE: corrected Appointment with Order -&gt; Appointement without Order</t>
   </si>
 </sst>
 </file>
@@ -4384,6 +4396,9 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -4401,9 +4416,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4770,14 +4782,14 @@
       <c r="C3" s="14"/>
     </row>
     <row r="4" spans="1:3" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="43" t="s">
         <v>60</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="16"/>
     </row>
     <row r="5" spans="1:3" ht="258" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="43"/>
+      <c r="A5" s="44"/>
       <c r="B5" s="19"/>
       <c r="C5" s="14"/>
     </row>
@@ -4789,17 +4801,17 @@
       <c r="C6" s="11"/>
     </row>
     <row r="7" spans="1:3" ht="98" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="45"/>
+      <c r="B7" s="46"/>
     </row>
     <row r="8" spans="1:3" ht="126" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
-      <c r="B8" s="46"/>
+      <c r="A8" s="45"/>
+      <c r="B8" s="47"/>
     </row>
     <row r="9" spans="1:3" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="42"/>
+      <c r="A9" s="43"/>
       <c r="B9" s="18"/>
     </row>
     <row r="10" spans="1:3" ht="292" x14ac:dyDescent="0.2">
@@ -4905,7 +4917,7 @@
         <v>23</v>
       </c>
       <c r="S1" s="36" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="T1" s="39" t="s">
         <v>24</v>
@@ -4948,7 +4960,7 @@
       </c>
       <c r="Q2" s="27"/>
       <c r="R2" s="27" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="S2" s="27" t="s">
         <v>68</v>
@@ -5064,7 +5076,7 @@
         <v>94</v>
       </c>
       <c r="R6" s="27" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="S6" s="27" t="s">
         <v>68</v>
@@ -5116,10 +5128,10 @@
         <v>94</v>
       </c>
       <c r="R8" s="27" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="S8" s="27" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="34" x14ac:dyDescent="0.2">
@@ -5194,7 +5206,7 @@
         <v>83</v>
       </c>
       <c r="S11" s="27" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="119" x14ac:dyDescent="0.2">
@@ -5292,7 +5304,7 @@
         <v>85</v>
       </c>
       <c r="S15" s="27" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="16" spans="1:32" ht="68" x14ac:dyDescent="0.2">
@@ -5367,10 +5379,10 @@
         <v>94</v>
       </c>
       <c r="R18" s="27" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="S18" s="27" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -5937,7 +5949,7 @@
         <v>98</v>
       </c>
       <c r="R42" s="27" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -5963,7 +5975,7 @@
         <v>98</v>
       </c>
       <c r="R43" s="27" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -5989,7 +6001,7 @@
         <v>98</v>
       </c>
       <c r="R44" s="27" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
     </row>
     <row r="45" spans="1:19" ht="85" x14ac:dyDescent="0.2">
@@ -6378,7 +6390,7 @@
         <v>190</v>
       </c>
       <c r="R60" s="27" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="S60" s="27" t="s">
         <v>68</v>
@@ -6706,7 +6718,7 @@
         <v>94</v>
       </c>
       <c r="R74" s="27" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="S74" s="27" t="s">
         <v>68</v>
@@ -6735,7 +6747,7 @@
         <v>98</v>
       </c>
       <c r="R75" s="27" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="S75" s="27" t="s">
         <v>68</v>
@@ -6787,7 +6799,7 @@
         <v>98</v>
       </c>
       <c r="R77" s="27" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="S77" s="27" t="s">
         <v>68</v>
@@ -6816,7 +6828,7 @@
         <v>94</v>
       </c>
       <c r="R78" s="27" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="S78" s="27" t="s">
         <v>68</v>
@@ -6824,7 +6836,7 @@
     </row>
     <row r="79" spans="1:19" ht="136" x14ac:dyDescent="0.2">
       <c r="A79" s="25" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="B79" s="32" t="s">
         <v>327</v>
@@ -6845,7 +6857,7 @@
         <v>94</v>
       </c>
       <c r="R79" s="27" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="S79" s="27" t="s">
         <v>68</v>
@@ -6853,13 +6865,13 @@
     </row>
     <row r="80" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="B80" s="32" t="s">
         <v>327</v>
       </c>
       <c r="C80" s="25" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="D80" s="25" t="s">
         <v>27</v>
@@ -6874,10 +6886,10 @@
         <v>94</v>
       </c>
       <c r="R80" s="27" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="S80" s="27" t="s">
-        <v>834</v>
+        <v>68</v>
       </c>
     </row>
     <row r="81" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -7018,10 +7030,10 @@
         <v>98</v>
       </c>
       <c r="R86" s="27" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="S86" s="27" t="s">
-        <v>834</v>
+        <v>68</v>
       </c>
     </row>
     <row r="87" spans="1:19" ht="68" x14ac:dyDescent="0.2">
@@ -7142,7 +7154,7 @@
         <v>94</v>
       </c>
       <c r="R91" s="27" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
     </row>
     <row r="92" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -7170,13 +7182,13 @@
     </row>
     <row r="93" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B93" s="32" t="s">
         <v>363</v>
       </c>
       <c r="C93" s="25" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="D93" s="25" t="s">
         <v>27</v>
@@ -7191,7 +7203,7 @@
         <v>94</v>
       </c>
       <c r="R93" s="27" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="S93" s="27" t="s">
         <v>68</v>
@@ -7199,13 +7211,13 @@
     </row>
     <row r="94" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B94" s="32" t="s">
         <v>363</v>
       </c>
       <c r="C94" s="25" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="D94" s="25" t="s">
         <v>27</v>
@@ -7220,7 +7232,7 @@
         <v>94</v>
       </c>
       <c r="R94" s="27" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="S94" s="27" t="s">
         <v>68</v>
@@ -7344,7 +7356,7 @@
         <v>98</v>
       </c>
       <c r="R99" s="27" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="S99" s="27" t="s">
         <v>68</v>
@@ -7373,7 +7385,7 @@
         <v>94</v>
       </c>
       <c r="R100" s="27" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="S100" s="27" t="s">
         <v>68</v>
@@ -7402,7 +7414,7 @@
         <v>94</v>
       </c>
       <c r="R101" s="27" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="S101" s="27" t="s">
         <v>68</v>
@@ -7670,7 +7682,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A113" s="25" t="s">
         <v>417</v>
       </c>
@@ -7693,7 +7705,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A114" s="25" t="s">
         <v>419</v>
       </c>
@@ -7716,7 +7728,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A115" s="25" t="s">
         <v>422</v>
       </c>
@@ -7739,7 +7751,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="102" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A116" s="25" t="s">
         <v>425</v>
       </c>
@@ -7762,7 +7774,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A117" s="25" t="s">
         <v>428</v>
       </c>
@@ -7785,7 +7797,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="102" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A118" s="25" t="s">
         <v>431</v>
       </c>
@@ -7808,7 +7820,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="153" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:19" ht="153" x14ac:dyDescent="0.2">
       <c r="A119" s="25" t="s">
         <v>434</v>
       </c>
@@ -7831,7 +7843,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A120" s="25" t="s">
         <v>437</v>
       </c>
@@ -7854,10 +7866,13 @@
         <v>94</v>
       </c>
       <c r="R120" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S120" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A121" s="25" t="s">
         <v>440</v>
       </c>
@@ -7880,10 +7895,13 @@
         <v>94</v>
       </c>
       <c r="R121" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S121" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A122" s="25" t="s">
         <v>443</v>
       </c>
@@ -7906,7 +7924,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A123" s="25" t="s">
         <v>446</v>
       </c>
@@ -7929,7 +7947,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A124" s="25" t="s">
         <v>449</v>
       </c>
@@ -7952,10 +7970,13 @@
         <v>94</v>
       </c>
       <c r="R124" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S124" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A125" s="25" t="s">
         <v>452</v>
       </c>
@@ -7978,7 +7999,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="102" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A126" s="25" t="s">
         <v>455</v>
       </c>
@@ -8001,10 +8022,13 @@
         <v>457</v>
       </c>
       <c r="R126" s="27" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="127" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+        <v>838</v>
+      </c>
+      <c r="S126" s="27" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="127" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A127" s="25" t="s">
         <v>459</v>
       </c>
@@ -8027,10 +8051,13 @@
         <v>94</v>
       </c>
       <c r="R127" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S127" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A128" s="25" t="s">
         <v>462</v>
       </c>
@@ -8053,7 +8080,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A129" s="25" t="s">
         <v>465</v>
       </c>
@@ -8076,10 +8103,13 @@
         <v>94</v>
       </c>
       <c r="R129" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S129" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A130" s="25" t="s">
         <v>468</v>
       </c>
@@ -8102,7 +8132,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A131" s="25" t="s">
         <v>471</v>
       </c>
@@ -8125,10 +8155,13 @@
         <v>94</v>
       </c>
       <c r="R131" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S131" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A132" s="25" t="s">
         <v>474</v>
       </c>
@@ -8151,7 +8184,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="102" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A133" s="25" t="s">
         <v>477</v>
       </c>
@@ -8174,10 +8207,13 @@
         <v>457</v>
       </c>
       <c r="R133" s="27" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="134" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+        <v>838</v>
+      </c>
+      <c r="S133" s="27" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="134" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A134" s="25" t="s">
         <v>480</v>
       </c>
@@ -8200,7 +8236,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A135" s="25" t="s">
         <v>483</v>
       </c>
@@ -8223,10 +8259,13 @@
         <v>94</v>
       </c>
       <c r="R135" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S135" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A136" s="25" t="s">
         <v>486</v>
       </c>
@@ -8249,7 +8288,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A137" s="25" t="s">
         <v>489</v>
       </c>
@@ -8272,10 +8311,13 @@
         <v>94</v>
       </c>
       <c r="R137" s="27" t="s">
+        <v>837</v>
+      </c>
+      <c r="S137" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A138" s="25" t="s">
         <v>492</v>
       </c>
@@ -8298,7 +8340,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="102" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A139" s="25" t="s">
         <v>495</v>
       </c>
@@ -8321,10 +8363,13 @@
         <v>457</v>
       </c>
       <c r="R139" s="27" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="140" spans="1:18" ht="51" x14ac:dyDescent="0.2">
+        <v>838</v>
+      </c>
+      <c r="S139" s="27" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="140" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A140" s="25" t="s">
         <v>498</v>
       </c>
@@ -8350,7 +8395,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A141" s="25" t="s">
         <v>501</v>
       </c>
@@ -8373,7 +8418,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A142" s="25" t="s">
         <v>504</v>
       </c>
@@ -8396,10 +8441,13 @@
         <v>94</v>
       </c>
       <c r="R142" s="27" t="s">
+        <v>839</v>
+      </c>
+      <c r="S142" s="27" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="68" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A143" s="25" t="s">
         <v>507</v>
       </c>
@@ -8422,7 +8470,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="85" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A144" s="25" t="s">
         <v>510</v>
       </c>
@@ -8445,7 +8493,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="145" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A145" s="25" t="s">
         <v>513</v>
       </c>
@@ -8468,7 +8516,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="146" spans="1:19" ht="85" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A146" s="25" t="s">
         <v>516</v>
       </c>
@@ -8491,7 +8539,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="147" spans="1:19" ht="187" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:21" ht="187" x14ac:dyDescent="0.2">
       <c r="A147" s="25" t="s">
         <v>519</v>
       </c>
@@ -8499,7 +8547,7 @@
         <v>520</v>
       </c>
       <c r="C147" s="25" t="s">
-        <v>521</v>
+        <v>840</v>
       </c>
       <c r="D147" s="25" t="s">
         <v>27</v>
@@ -8514,21 +8562,24 @@
         <v>94</v>
       </c>
       <c r="R147" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S147" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="148" spans="1:19" ht="170" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+      <c r="U147" s="27" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="148" spans="1:21" ht="170" x14ac:dyDescent="0.2">
       <c r="A148" s="25" t="s">
+        <v>521</v>
+      </c>
+      <c r="B148" s="32" t="s">
         <v>522</v>
       </c>
-      <c r="B148" s="32" t="s">
-        <v>523</v>
-      </c>
       <c r="C148" s="25" t="s">
-        <v>524</v>
+        <v>841</v>
       </c>
       <c r="D148" s="25" t="s">
         <v>27</v>
@@ -8543,18 +8594,21 @@
         <v>94</v>
       </c>
       <c r="R148" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S148" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="149" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+      <c r="U148" s="27" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="149" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A149" s="25" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="B149" s="32" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C149" s="25" t="s">
         <v>71</v>
@@ -8572,21 +8626,21 @@
         <v>94</v>
       </c>
       <c r="R149" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S149" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="150" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="150" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A150" s="25" t="s">
+        <v>525</v>
+      </c>
+      <c r="B150" s="32" t="s">
+        <v>526</v>
+      </c>
+      <c r="C150" s="25" t="s">
         <v>527</v>
-      </c>
-      <c r="B150" s="32" t="s">
-        <v>528</v>
-      </c>
-      <c r="C150" s="25" t="s">
-        <v>529</v>
       </c>
       <c r="D150" s="25" t="s">
         <v>27</v>
@@ -8601,21 +8655,21 @@
         <v>94</v>
       </c>
       <c r="R150" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S150" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="151" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="151" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A151" s="25" t="s">
+        <v>528</v>
+      </c>
+      <c r="B151" s="32" t="s">
+        <v>529</v>
+      </c>
+      <c r="C151" s="25" t="s">
         <v>530</v>
-      </c>
-      <c r="B151" s="32" t="s">
-        <v>531</v>
-      </c>
-      <c r="C151" s="25" t="s">
-        <v>532</v>
       </c>
       <c r="D151" s="25" t="s">
         <v>27</v>
@@ -8630,18 +8684,18 @@
         <v>94</v>
       </c>
       <c r="R151" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S151" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="152" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="152" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A152" s="25" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="B152" s="32" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C152" s="25" t="s">
         <v>72</v>
@@ -8659,18 +8713,18 @@
         <v>94</v>
       </c>
       <c r="R152" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S152" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="153" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="153" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A153" s="25" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="B153" s="32" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C153" s="25" t="s">
         <v>73</v>
@@ -8688,21 +8742,21 @@
         <v>94</v>
       </c>
       <c r="R153" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S153" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="154" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="154" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A154" s="25" t="s">
+        <v>535</v>
+      </c>
+      <c r="B154" s="32" t="s">
+        <v>536</v>
+      </c>
+      <c r="C154" s="25" t="s">
         <v>537</v>
-      </c>
-      <c r="B154" s="32" t="s">
-        <v>538</v>
-      </c>
-      <c r="C154" s="25" t="s">
-        <v>539</v>
       </c>
       <c r="D154" s="25" t="s">
         <v>27</v>
@@ -8717,18 +8771,18 @@
         <v>94</v>
       </c>
       <c r="R154" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S154" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="155" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="155" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A155" s="25" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="B155" s="32" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C155" s="25" t="s">
         <v>74</v>
@@ -8746,18 +8800,18 @@
         <v>94</v>
       </c>
       <c r="R155" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S155" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="156" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="156" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A156" s="25" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="B156" s="32" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C156" s="25" t="s">
         <v>75</v>
@@ -8775,18 +8829,18 @@
         <v>94</v>
       </c>
       <c r="R156" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S156" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="157" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="157" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A157" s="25" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="B157" s="32" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C157" s="25" t="s">
         <v>76</v>
@@ -8804,18 +8858,18 @@
         <v>94</v>
       </c>
       <c r="R157" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S157" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="158" spans="1:19" ht="68" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="158" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A158" s="25" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="B158" s="32" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C158" s="25" t="s">
         <v>77</v>
@@ -8833,21 +8887,21 @@
         <v>94</v>
       </c>
       <c r="R158" s="27" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="S158" s="27" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="159" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="159" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A159" s="25" t="s">
+        <v>546</v>
+      </c>
+      <c r="B159" s="32" t="s">
+        <v>547</v>
+      </c>
+      <c r="C159" s="25" t="s">
         <v>548</v>
-      </c>
-      <c r="B159" s="32" t="s">
-        <v>549</v>
-      </c>
-      <c r="C159" s="25" t="s">
-        <v>550</v>
       </c>
       <c r="D159" s="25" t="s">
         <v>27</v>
@@ -8868,15 +8922,15 @@
         <v>68</v>
       </c>
     </row>
-    <row r="160" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A160" s="25" t="s">
+        <v>549</v>
+      </c>
+      <c r="B160" s="32" t="s">
+        <v>550</v>
+      </c>
+      <c r="C160" s="25" t="s">
         <v>551</v>
-      </c>
-      <c r="B160" s="32" t="s">
-        <v>552</v>
-      </c>
-      <c r="C160" s="25" t="s">
-        <v>553</v>
       </c>
       <c r="D160" s="25" t="s">
         <v>26</v>
@@ -8893,13 +8947,13 @@
     </row>
     <row r="161" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A161" s="25" t="s">
+        <v>552</v>
+      </c>
+      <c r="B161" s="32" t="s">
+        <v>553</v>
+      </c>
+      <c r="C161" s="25" t="s">
         <v>554</v>
-      </c>
-      <c r="B161" s="32" t="s">
-        <v>555</v>
-      </c>
-      <c r="C161" s="25" t="s">
-        <v>556</v>
       </c>
       <c r="D161" s="25" t="s">
         <v>28</v>
@@ -8916,13 +8970,13 @@
     </row>
     <row r="162" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A162" s="25" t="s">
+        <v>555</v>
+      </c>
+      <c r="B162" s="32" t="s">
+        <v>556</v>
+      </c>
+      <c r="C162" s="25" t="s">
         <v>557</v>
-      </c>
-      <c r="B162" s="32" t="s">
-        <v>558</v>
-      </c>
-      <c r="C162" s="25" t="s">
-        <v>559</v>
       </c>
       <c r="D162" s="25" t="s">
         <v>28</v>
@@ -8939,13 +8993,13 @@
     </row>
     <row r="163" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A163" s="25" t="s">
+        <v>558</v>
+      </c>
+      <c r="B163" s="32" t="s">
+        <v>559</v>
+      </c>
+      <c r="C163" s="25" t="s">
         <v>560</v>
-      </c>
-      <c r="B163" s="32" t="s">
-        <v>561</v>
-      </c>
-      <c r="C163" s="25" t="s">
-        <v>562</v>
       </c>
       <c r="D163" s="25" t="s">
         <v>28</v>
@@ -8962,13 +9016,13 @@
     </row>
     <row r="164" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A164" s="25" t="s">
+        <v>561</v>
+      </c>
+      <c r="B164" s="32" t="s">
+        <v>562</v>
+      </c>
+      <c r="C164" s="25" t="s">
         <v>563</v>
-      </c>
-      <c r="B164" s="32" t="s">
-        <v>564</v>
-      </c>
-      <c r="C164" s="25" t="s">
-        <v>565</v>
       </c>
       <c r="D164" s="25" t="s">
         <v>27</v>
@@ -8985,13 +9039,13 @@
     </row>
     <row r="165" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A165" s="25" t="s">
+        <v>564</v>
+      </c>
+      <c r="B165" s="32" t="s">
+        <v>565</v>
+      </c>
+      <c r="C165" s="25" t="s">
         <v>566</v>
-      </c>
-      <c r="B165" s="32" t="s">
-        <v>567</v>
-      </c>
-      <c r="C165" s="25" t="s">
-        <v>568</v>
       </c>
       <c r="D165" s="25" t="s">
         <v>27</v>
@@ -9008,13 +9062,13 @@
     </row>
     <row r="166" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A166" s="25" t="s">
+        <v>567</v>
+      </c>
+      <c r="B166" s="32" t="s">
+        <v>568</v>
+      </c>
+      <c r="C166" s="25" t="s">
         <v>569</v>
-      </c>
-      <c r="B166" s="32" t="s">
-        <v>570</v>
-      </c>
-      <c r="C166" s="25" t="s">
-        <v>571</v>
       </c>
       <c r="D166" s="25" t="s">
         <v>27</v>
@@ -9031,13 +9085,13 @@
     </row>
     <row r="167" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A167" s="25" t="s">
+        <v>570</v>
+      </c>
+      <c r="B167" s="32" t="s">
+        <v>571</v>
+      </c>
+      <c r="C167" s="25" t="s">
         <v>572</v>
-      </c>
-      <c r="B167" s="32" t="s">
-        <v>573</v>
-      </c>
-      <c r="C167" s="25" t="s">
-        <v>574</v>
       </c>
       <c r="D167" s="25" t="s">
         <v>28</v>
@@ -9054,13 +9108,13 @@
     </row>
     <row r="168" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A168" s="25" t="s">
+        <v>573</v>
+      </c>
+      <c r="B168" s="32" t="s">
+        <v>574</v>
+      </c>
+      <c r="C168" s="25" t="s">
         <v>575</v>
-      </c>
-      <c r="B168" s="32" t="s">
-        <v>576</v>
-      </c>
-      <c r="C168" s="25" t="s">
-        <v>577</v>
       </c>
       <c r="D168" s="25" t="s">
         <v>28</v>
@@ -9077,13 +9131,13 @@
     </row>
     <row r="169" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A169" s="25" t="s">
+        <v>576</v>
+      </c>
+      <c r="B169" s="32" t="s">
+        <v>577</v>
+      </c>
+      <c r="C169" s="25" t="s">
         <v>578</v>
-      </c>
-      <c r="B169" s="32" t="s">
-        <v>579</v>
-      </c>
-      <c r="C169" s="25" t="s">
-        <v>580</v>
       </c>
       <c r="D169" s="25" t="s">
         <v>28</v>
@@ -9100,13 +9154,13 @@
     </row>
     <row r="170" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A170" s="25" t="s">
+        <v>579</v>
+      </c>
+      <c r="B170" s="32" t="s">
+        <v>580</v>
+      </c>
+      <c r="C170" s="25" t="s">
         <v>581</v>
-      </c>
-      <c r="B170" s="32" t="s">
-        <v>582</v>
-      </c>
-      <c r="C170" s="25" t="s">
-        <v>583</v>
       </c>
       <c r="D170" s="25" t="s">
         <v>28</v>
@@ -9123,13 +9177,13 @@
     </row>
     <row r="171" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A171" s="25" t="s">
+        <v>582</v>
+      </c>
+      <c r="B171" s="32" t="s">
+        <v>583</v>
+      </c>
+      <c r="C171" s="25" t="s">
         <v>584</v>
-      </c>
-      <c r="B171" s="32" t="s">
-        <v>585</v>
-      </c>
-      <c r="C171" s="25" t="s">
-        <v>586</v>
       </c>
       <c r="D171" s="25" t="s">
         <v>28</v>
@@ -9146,13 +9200,13 @@
     </row>
     <row r="172" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A172" s="25" t="s">
+        <v>585</v>
+      </c>
+      <c r="B172" s="32" t="s">
+        <v>586</v>
+      </c>
+      <c r="C172" s="25" t="s">
         <v>587</v>
-      </c>
-      <c r="B172" s="32" t="s">
-        <v>588</v>
-      </c>
-      <c r="C172" s="25" t="s">
-        <v>589</v>
       </c>
       <c r="D172" s="25" t="s">
         <v>28</v>
@@ -9169,13 +9223,13 @@
     </row>
     <row r="173" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A173" s="25" t="s">
+        <v>588</v>
+      </c>
+      <c r="B173" s="32" t="s">
+        <v>589</v>
+      </c>
+      <c r="C173" s="25" t="s">
         <v>590</v>
-      </c>
-      <c r="B173" s="32" t="s">
-        <v>591</v>
-      </c>
-      <c r="C173" s="25" t="s">
-        <v>592</v>
       </c>
       <c r="D173" s="25" t="s">
         <v>29</v>
@@ -9192,13 +9246,13 @@
     </row>
     <row r="174" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A174" s="25" t="s">
+        <v>591</v>
+      </c>
+      <c r="B174" s="32" t="s">
+        <v>592</v>
+      </c>
+      <c r="C174" s="25" t="s">
         <v>593</v>
-      </c>
-      <c r="B174" s="32" t="s">
-        <v>594</v>
-      </c>
-      <c r="C174" s="25" t="s">
-        <v>595</v>
       </c>
       <c r="D174" s="25" t="s">
         <v>27</v>
@@ -9215,13 +9269,13 @@
     </row>
     <row r="175" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A175" s="25" t="s">
+        <v>594</v>
+      </c>
+      <c r="B175" s="32" t="s">
+        <v>595</v>
+      </c>
+      <c r="C175" s="25" t="s">
         <v>596</v>
-      </c>
-      <c r="B175" s="32" t="s">
-        <v>597</v>
-      </c>
-      <c r="C175" s="25" t="s">
-        <v>598</v>
       </c>
       <c r="D175" s="25" t="s">
         <v>27</v>
@@ -9236,7 +9290,7 @@
         <v>94</v>
       </c>
       <c r="R175" s="27" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="S175" s="27" t="s">
         <v>68</v>
@@ -9244,13 +9298,13 @@
     </row>
     <row r="176" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A176" s="25" t="s">
+        <v>597</v>
+      </c>
+      <c r="B176" s="32" t="s">
+        <v>598</v>
+      </c>
+      <c r="C176" s="25" t="s">
         <v>599</v>
-      </c>
-      <c r="B176" s="32" t="s">
-        <v>600</v>
-      </c>
-      <c r="C176" s="25" t="s">
-        <v>601</v>
       </c>
       <c r="D176" s="25" t="s">
         <v>28</v>
@@ -9267,13 +9321,13 @@
     </row>
     <row r="177" spans="1:22" ht="85" x14ac:dyDescent="0.2">
       <c r="A177" s="25" t="s">
+        <v>600</v>
+      </c>
+      <c r="B177" s="32" t="s">
+        <v>601</v>
+      </c>
+      <c r="C177" s="25" t="s">
         <v>602</v>
-      </c>
-      <c r="B177" s="32" t="s">
-        <v>603</v>
-      </c>
-      <c r="C177" s="25" t="s">
-        <v>604</v>
       </c>
       <c r="D177" s="25" t="s">
         <v>28</v>
@@ -9290,13 +9344,13 @@
     </row>
     <row r="178" spans="1:22" ht="51" x14ac:dyDescent="0.2">
       <c r="A178" s="25" t="s">
+        <v>603</v>
+      </c>
+      <c r="B178" s="32" t="s">
+        <v>604</v>
+      </c>
+      <c r="C178" s="25" t="s">
         <v>605</v>
-      </c>
-      <c r="B178" s="32" t="s">
-        <v>606</v>
-      </c>
-      <c r="C178" s="25" t="s">
-        <v>607</v>
       </c>
       <c r="D178" s="25" t="s">
         <v>30</v>
@@ -9313,13 +9367,13 @@
     </row>
     <row r="179" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A179" s="25" t="s">
+        <v>606</v>
+      </c>
+      <c r="B179" s="32" t="s">
+        <v>607</v>
+      </c>
+      <c r="C179" s="25" t="s">
         <v>608</v>
-      </c>
-      <c r="B179" s="32" t="s">
-        <v>609</v>
-      </c>
-      <c r="C179" s="25" t="s">
-        <v>610</v>
       </c>
       <c r="D179" s="25" t="s">
         <v>27</v>
@@ -9336,13 +9390,13 @@
     </row>
     <row r="180" spans="1:22" ht="17" x14ac:dyDescent="0.2">
       <c r="A180" s="25" t="s">
+        <v>609</v>
+      </c>
+      <c r="B180" s="32" t="s">
+        <v>610</v>
+      </c>
+      <c r="C180" s="25" t="s">
         <v>611</v>
-      </c>
-      <c r="B180" s="32" t="s">
-        <v>612</v>
-      </c>
-      <c r="C180" s="25" t="s">
-        <v>613</v>
       </c>
       <c r="D180" s="25" t="s">
         <v>27</v>
@@ -9359,13 +9413,13 @@
     </row>
     <row r="181" spans="1:22" ht="51" x14ac:dyDescent="0.2">
       <c r="A181" s="25" t="s">
+        <v>612</v>
+      </c>
+      <c r="B181" s="32" t="s">
+        <v>613</v>
+      </c>
+      <c r="C181" s="25" t="s">
         <v>614</v>
-      </c>
-      <c r="B181" s="32" t="s">
-        <v>615</v>
-      </c>
-      <c r="C181" s="25" t="s">
-        <v>616</v>
       </c>
       <c r="D181" s="25" t="s">
         <v>28</v>
@@ -9382,13 +9436,13 @@
     </row>
     <row r="182" spans="1:22" ht="68" x14ac:dyDescent="0.2">
       <c r="A182" s="25" t="s">
+        <v>615</v>
+      </c>
+      <c r="B182" s="32" t="s">
+        <v>616</v>
+      </c>
+      <c r="C182" s="25" t="s">
         <v>617</v>
-      </c>
-      <c r="B182" s="32" t="s">
-        <v>618</v>
-      </c>
-      <c r="C182" s="25" t="s">
-        <v>619</v>
       </c>
       <c r="D182" s="25" t="s">
         <v>28</v>
@@ -9405,13 +9459,13 @@
     </row>
     <row r="183" spans="1:22" ht="85" x14ac:dyDescent="0.2">
       <c r="A183" s="25" t="s">
+        <v>618</v>
+      </c>
+      <c r="B183" s="32" t="s">
+        <v>619</v>
+      </c>
+      <c r="C183" s="25" t="s">
         <v>620</v>
-      </c>
-      <c r="B183" s="32" t="s">
-        <v>621</v>
-      </c>
-      <c r="C183" s="25" t="s">
-        <v>622</v>
       </c>
       <c r="D183" s="25" t="s">
         <v>27</v>
@@ -9428,13 +9482,13 @@
     </row>
     <row r="184" spans="1:22" ht="102" x14ac:dyDescent="0.2">
       <c r="A184" s="25" t="s">
+        <v>621</v>
+      </c>
+      <c r="B184" s="32" t="s">
+        <v>622</v>
+      </c>
+      <c r="C184" s="25" t="s">
         <v>623</v>
-      </c>
-      <c r="B184" s="32" t="s">
-        <v>624</v>
-      </c>
-      <c r="C184" s="25" t="s">
-        <v>625</v>
       </c>
       <c r="D184" s="25" t="s">
         <v>30</v>
@@ -9451,13 +9505,13 @@
     </row>
     <row r="185" spans="1:22" ht="68" x14ac:dyDescent="0.2">
       <c r="A185" s="25" t="s">
+        <v>624</v>
+      </c>
+      <c r="B185" s="32" t="s">
+        <v>625</v>
+      </c>
+      <c r="C185" s="25" t="s">
         <v>626</v>
-      </c>
-      <c r="B185" s="32" t="s">
-        <v>627</v>
-      </c>
-      <c r="C185" s="25" t="s">
-        <v>628</v>
       </c>
       <c r="D185" s="25" t="s">
         <v>27</v>
@@ -9474,13 +9528,13 @@
     </row>
     <row r="186" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A186" s="25" t="s">
+        <v>627</v>
+      </c>
+      <c r="B186" s="32" t="s">
+        <v>628</v>
+      </c>
+      <c r="C186" s="25" t="s">
         <v>629</v>
-      </c>
-      <c r="B186" s="32" t="s">
-        <v>630</v>
-      </c>
-      <c r="C186" s="25" t="s">
-        <v>631</v>
       </c>
       <c r="D186" s="25" t="s">
         <v>30</v>
@@ -9497,13 +9551,13 @@
     </row>
     <row r="187" spans="1:22" ht="51" x14ac:dyDescent="0.2">
       <c r="A187" s="25" t="s">
+        <v>630</v>
+      </c>
+      <c r="B187" s="32" t="s">
+        <v>631</v>
+      </c>
+      <c r="C187" s="25" t="s">
         <v>632</v>
-      </c>
-      <c r="B187" s="32" t="s">
-        <v>633</v>
-      </c>
-      <c r="C187" s="25" t="s">
-        <v>634</v>
       </c>
       <c r="D187" s="25" t="s">
         <v>27</v>
@@ -9520,13 +9574,13 @@
     </row>
     <row r="188" spans="1:22" ht="34" x14ac:dyDescent="0.2">
       <c r="A188" s="25" t="s">
+        <v>633</v>
+      </c>
+      <c r="B188" s="32" t="s">
+        <v>634</v>
+      </c>
+      <c r="C188" s="25" t="s">
         <v>635</v>
-      </c>
-      <c r="B188" s="32" t="s">
-        <v>636</v>
-      </c>
-      <c r="C188" s="25" t="s">
-        <v>637</v>
       </c>
       <c r="D188" s="25" t="s">
         <v>26</v>
@@ -9544,13 +9598,13 @@
     </row>
     <row r="189" spans="1:22" ht="51" x14ac:dyDescent="0.2">
       <c r="A189" s="25" t="s">
+        <v>636</v>
+      </c>
+      <c r="B189" s="32" t="s">
+        <v>637</v>
+      </c>
+      <c r="C189" s="25" t="s">
         <v>638</v>
-      </c>
-      <c r="B189" s="32" t="s">
-        <v>639</v>
-      </c>
-      <c r="C189" s="25" t="s">
-        <v>640</v>
       </c>
       <c r="D189" s="25" t="s">
         <v>27</v>
@@ -9567,13 +9621,13 @@
     </row>
     <row r="190" spans="1:22" ht="85" x14ac:dyDescent="0.2">
       <c r="A190" s="25" t="s">
+        <v>639</v>
+      </c>
+      <c r="B190" s="32" t="s">
+        <v>640</v>
+      </c>
+      <c r="C190" s="25" t="s">
         <v>641</v>
-      </c>
-      <c r="B190" s="32" t="s">
-        <v>642</v>
-      </c>
-      <c r="C190" s="25" t="s">
-        <v>643</v>
       </c>
       <c r="D190" s="25" t="s">
         <v>27</v>
@@ -9590,13 +9644,13 @@
     </row>
     <row r="191" spans="1:22" ht="51" x14ac:dyDescent="0.2">
       <c r="A191" s="25" t="s">
+        <v>642</v>
+      </c>
+      <c r="B191" s="32" t="s">
+        <v>643</v>
+      </c>
+      <c r="C191" s="25" t="s">
         <v>644</v>
-      </c>
-      <c r="B191" s="32" t="s">
-        <v>645</v>
-      </c>
-      <c r="C191" s="25" t="s">
-        <v>646</v>
       </c>
       <c r="D191" s="25" t="s">
         <v>27</v>
@@ -9613,13 +9667,13 @@
     </row>
     <row r="192" spans="1:22" ht="136" x14ac:dyDescent="0.2">
       <c r="A192" s="25" t="s">
+        <v>645</v>
+      </c>
+      <c r="B192" s="32" t="s">
+        <v>646</v>
+      </c>
+      <c r="C192" s="25" t="s">
         <v>647</v>
-      </c>
-      <c r="B192" s="32" t="s">
-        <v>648</v>
-      </c>
-      <c r="C192" s="25" t="s">
-        <v>649</v>
       </c>
       <c r="D192" s="25" t="s">
         <v>27</v>
@@ -9639,13 +9693,13 @@
     </row>
     <row r="193" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A193" s="25" t="s">
+        <v>648</v>
+      </c>
+      <c r="B193" s="32" t="s">
+        <v>649</v>
+      </c>
+      <c r="C193" s="25" t="s">
         <v>650</v>
-      </c>
-      <c r="B193" s="32" t="s">
-        <v>651</v>
-      </c>
-      <c r="C193" s="25" t="s">
-        <v>652</v>
       </c>
       <c r="D193" s="25" t="s">
         <v>27</v>
@@ -9662,13 +9716,13 @@
     </row>
     <row r="194" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A194" s="25" t="s">
+        <v>651</v>
+      </c>
+      <c r="B194" s="32" t="s">
+        <v>652</v>
+      </c>
+      <c r="C194" s="25" t="s">
         <v>653</v>
-      </c>
-      <c r="B194" s="32" t="s">
-        <v>654</v>
-      </c>
-      <c r="C194" s="25" t="s">
-        <v>655</v>
       </c>
       <c r="D194" s="25" t="s">
         <v>26</v>
@@ -9685,13 +9739,13 @@
     </row>
     <row r="195" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A195" s="25" t="s">
+        <v>654</v>
+      </c>
+      <c r="B195" s="32" t="s">
+        <v>655</v>
+      </c>
+      <c r="C195" s="25" t="s">
         <v>656</v>
-      </c>
-      <c r="B195" s="32" t="s">
-        <v>657</v>
-      </c>
-      <c r="C195" s="25" t="s">
-        <v>658</v>
       </c>
       <c r="D195" s="25" t="s">
         <v>26</v>
@@ -9708,13 +9762,13 @@
     </row>
     <row r="196" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A196" s="25" t="s">
+        <v>657</v>
+      </c>
+      <c r="B196" s="32" t="s">
+        <v>658</v>
+      </c>
+      <c r="C196" s="25" t="s">
         <v>659</v>
-      </c>
-      <c r="B196" s="32" t="s">
-        <v>660</v>
-      </c>
-      <c r="C196" s="25" t="s">
-        <v>661</v>
       </c>
       <c r="D196" s="25" t="s">
         <v>30</v>
@@ -9731,13 +9785,13 @@
     </row>
     <row r="197" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A197" s="25" t="s">
+        <v>660</v>
+      </c>
+      <c r="B197" s="32" t="s">
+        <v>661</v>
+      </c>
+      <c r="C197" s="25" t="s">
         <v>662</v>
-      </c>
-      <c r="B197" s="32" t="s">
-        <v>663</v>
-      </c>
-      <c r="C197" s="25" t="s">
-        <v>664</v>
       </c>
       <c r="D197" s="25" t="s">
         <v>28</v>
@@ -9754,13 +9808,13 @@
     </row>
     <row r="198" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A198" s="25" t="s">
+        <v>663</v>
+      </c>
+      <c r="B198" s="32" t="s">
+        <v>664</v>
+      </c>
+      <c r="C198" s="25" t="s">
         <v>665</v>
-      </c>
-      <c r="B198" s="32" t="s">
-        <v>666</v>
-      </c>
-      <c r="C198" s="25" t="s">
-        <v>667</v>
       </c>
       <c r="D198" s="25" t="s">
         <v>30</v>
@@ -9777,13 +9831,13 @@
     </row>
     <row r="199" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A199" s="25" t="s">
+        <v>666</v>
+      </c>
+      <c r="B199" s="32" t="s">
+        <v>667</v>
+      </c>
+      <c r="C199" s="25" t="s">
         <v>668</v>
-      </c>
-      <c r="B199" s="32" t="s">
-        <v>669</v>
-      </c>
-      <c r="C199" s="25" t="s">
-        <v>670</v>
       </c>
       <c r="D199" s="25" t="s">
         <v>28</v>
@@ -9800,13 +9854,13 @@
     </row>
     <row r="200" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A200" s="25" t="s">
+        <v>669</v>
+      </c>
+      <c r="B200" s="32" t="s">
+        <v>670</v>
+      </c>
+      <c r="C200" s="25" t="s">
         <v>671</v>
-      </c>
-      <c r="B200" s="32" t="s">
-        <v>672</v>
-      </c>
-      <c r="C200" s="25" t="s">
-        <v>673</v>
       </c>
       <c r="D200" s="25" t="s">
         <v>28</v>
@@ -9823,13 +9877,13 @@
     </row>
     <row r="201" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A201" s="25" t="s">
+        <v>672</v>
+      </c>
+      <c r="B201" s="32" t="s">
+        <v>673</v>
+      </c>
+      <c r="C201" s="25" t="s">
         <v>674</v>
-      </c>
-      <c r="B201" s="32" t="s">
-        <v>675</v>
-      </c>
-      <c r="C201" s="25" t="s">
-        <v>676</v>
       </c>
       <c r="D201" s="25" t="s">
         <v>27</v>
@@ -9849,13 +9903,13 @@
     </row>
     <row r="202" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A202" s="25" t="s">
+        <v>675</v>
+      </c>
+      <c r="B202" s="32" t="s">
+        <v>676</v>
+      </c>
+      <c r="C202" s="25" t="s">
         <v>677</v>
-      </c>
-      <c r="B202" s="32" t="s">
-        <v>678</v>
-      </c>
-      <c r="C202" s="25" t="s">
-        <v>679</v>
       </c>
       <c r="D202" s="25" t="s">
         <v>28</v>
@@ -9872,13 +9926,13 @@
     </row>
     <row r="203" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A203" s="25" t="s">
+        <v>678</v>
+      </c>
+      <c r="B203" s="32" t="s">
+        <v>679</v>
+      </c>
+      <c r="C203" s="25" t="s">
         <v>680</v>
-      </c>
-      <c r="B203" s="32" t="s">
-        <v>681</v>
-      </c>
-      <c r="C203" s="25" t="s">
-        <v>682</v>
       </c>
       <c r="D203" s="25" t="s">
         <v>28</v>
@@ -9895,13 +9949,13 @@
     </row>
     <row r="204" spans="1:19" ht="170" x14ac:dyDescent="0.2">
       <c r="A204" s="25" t="s">
+        <v>681</v>
+      </c>
+      <c r="B204" s="32" t="s">
+        <v>682</v>
+      </c>
+      <c r="C204" s="25" t="s">
         <v>683</v>
-      </c>
-      <c r="B204" s="32" t="s">
-        <v>684</v>
-      </c>
-      <c r="C204" s="25" t="s">
-        <v>685</v>
       </c>
       <c r="D204" s="25" t="s">
         <v>27</v>
@@ -9918,13 +9972,13 @@
     </row>
     <row r="205" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A205" s="25" t="s">
+        <v>684</v>
+      </c>
+      <c r="B205" s="32" t="s">
+        <v>685</v>
+      </c>
+      <c r="C205" s="25" t="s">
         <v>686</v>
-      </c>
-      <c r="B205" s="32" t="s">
-        <v>687</v>
-      </c>
-      <c r="C205" s="25" t="s">
-        <v>688</v>
       </c>
       <c r="D205" s="25" t="s">
         <v>27</v>
@@ -9941,13 +9995,13 @@
     </row>
     <row r="206" spans="1:19" ht="170" x14ac:dyDescent="0.2">
       <c r="A206" s="25" t="s">
+        <v>687</v>
+      </c>
+      <c r="B206" s="32" t="s">
+        <v>688</v>
+      </c>
+      <c r="C206" s="25" t="s">
         <v>689</v>
-      </c>
-      <c r="B206" s="32" t="s">
-        <v>690</v>
-      </c>
-      <c r="C206" s="25" t="s">
-        <v>691</v>
       </c>
       <c r="D206" s="25" t="s">
         <v>27</v>
@@ -9964,13 +10018,13 @@
     </row>
     <row r="207" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A207" s="25" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B207" s="32" t="s">
+        <v>691</v>
+      </c>
+      <c r="C207" s="25" t="s">
         <v>693</v>
-      </c>
-      <c r="C207" s="25" t="s">
-        <v>695</v>
       </c>
       <c r="D207" s="25" t="s">
         <v>27</v>
@@ -9982,10 +10036,10 @@
         <v>1</v>
       </c>
       <c r="P207" s="27" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="R207" s="27" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="S207" s="27" t="s">
         <v>68</v>
@@ -9993,10 +10047,10 @@
     </row>
     <row r="208" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A208" s="25" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="B208" s="32" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="C208" s="25" t="s">
         <v>78</v>
@@ -10016,13 +10070,13 @@
     </row>
     <row r="209" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A209" s="25" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B209" s="32" t="s">
+        <v>697</v>
+      </c>
+      <c r="C209" s="25" t="s">
         <v>699</v>
-      </c>
-      <c r="C209" s="25" t="s">
-        <v>701</v>
       </c>
       <c r="D209" s="25" t="s">
         <v>27</v>
@@ -10034,7 +10088,7 @@
         <v>0</v>
       </c>
       <c r="P209" s="27" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="R209" s="27" t="s">
         <v>90</v>
@@ -10042,13 +10096,13 @@
     </row>
     <row r="210" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A210" s="25" t="s">
+        <v>700</v>
+      </c>
+      <c r="B210" s="32" t="s">
+        <v>701</v>
+      </c>
+      <c r="C210" s="25" t="s">
         <v>702</v>
-      </c>
-      <c r="B210" s="32" t="s">
-        <v>703</v>
-      </c>
-      <c r="C210" s="25" t="s">
-        <v>704</v>
       </c>
       <c r="D210" s="25" t="s">
         <v>27</v>
@@ -10066,18 +10120,18 @@
         <v>91</v>
       </c>
       <c r="S210" s="27" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
     </row>
     <row r="211" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A211" s="25" t="s">
+        <v>703</v>
+      </c>
+      <c r="B211" s="32" t="s">
+        <v>704</v>
+      </c>
+      <c r="C211" s="25" t="s">
         <v>705</v>
-      </c>
-      <c r="B211" s="32" t="s">
-        <v>706</v>
-      </c>
-      <c r="C211" s="25" t="s">
-        <v>707</v>
       </c>
       <c r="D211" s="25" t="s">
         <v>26</v>
@@ -10094,13 +10148,13 @@
     </row>
     <row r="212" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A212" s="25" t="s">
+        <v>706</v>
+      </c>
+      <c r="B212" s="32" t="s">
+        <v>707</v>
+      </c>
+      <c r="C212" s="25" t="s">
         <v>708</v>
-      </c>
-      <c r="B212" s="32" t="s">
-        <v>709</v>
-      </c>
-      <c r="C212" s="25" t="s">
-        <v>710</v>
       </c>
       <c r="D212" s="25" t="s">
         <v>28</v>
@@ -10117,13 +10171,13 @@
     </row>
     <row r="213" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A213" s="25" t="s">
+        <v>709</v>
+      </c>
+      <c r="B213" s="32" t="s">
+        <v>710</v>
+      </c>
+      <c r="C213" s="25" t="s">
         <v>711</v>
-      </c>
-      <c r="B213" s="32" t="s">
-        <v>712</v>
-      </c>
-      <c r="C213" s="25" t="s">
-        <v>713</v>
       </c>
       <c r="D213" s="25" t="s">
         <v>27</v>
@@ -10140,13 +10194,13 @@
     </row>
     <row r="214" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A214" s="25" t="s">
+        <v>712</v>
+      </c>
+      <c r="B214" s="32" t="s">
+        <v>713</v>
+      </c>
+      <c r="C214" s="25" t="s">
         <v>714</v>
-      </c>
-      <c r="B214" s="32" t="s">
-        <v>715</v>
-      </c>
-      <c r="C214" s="25" t="s">
-        <v>716</v>
       </c>
       <c r="D214" s="25" t="s">
         <v>28</v>
@@ -10163,13 +10217,13 @@
     </row>
     <row r="215" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A215" s="25" t="s">
+        <v>715</v>
+      </c>
+      <c r="B215" s="32" t="s">
+        <v>716</v>
+      </c>
+      <c r="C215" s="25" t="s">
         <v>717</v>
-      </c>
-      <c r="B215" s="32" t="s">
-        <v>718</v>
-      </c>
-      <c r="C215" s="25" t="s">
-        <v>719</v>
       </c>
       <c r="D215" s="25" t="s">
         <v>28</v>
@@ -10186,10 +10240,10 @@
     </row>
     <row r="216" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A216" s="25" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B216" s="32" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C216" s="25" t="s">
         <v>79</v>
@@ -10209,13 +10263,13 @@
     </row>
     <row r="217" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A217" s="25" t="s">
+        <v>720</v>
+      </c>
+      <c r="B217" s="32" t="s">
+        <v>721</v>
+      </c>
+      <c r="C217" s="25" t="s">
         <v>722</v>
-      </c>
-      <c r="B217" s="32" t="s">
-        <v>723</v>
-      </c>
-      <c r="C217" s="25" t="s">
-        <v>724</v>
       </c>
       <c r="D217" s="25" t="s">
         <v>27</v>
@@ -10232,10 +10286,10 @@
     </row>
     <row r="218" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A218" s="25" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="B218" s="32" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="C218" s="25" t="s">
         <v>80</v>
@@ -10255,13 +10309,13 @@
     </row>
     <row r="219" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A219" s="25" t="s">
+        <v>725</v>
+      </c>
+      <c r="B219" s="32" t="s">
+        <v>726</v>
+      </c>
+      <c r="C219" s="25" t="s">
         <v>727</v>
-      </c>
-      <c r="B219" s="32" t="s">
-        <v>728</v>
-      </c>
-      <c r="C219" s="25" t="s">
-        <v>729</v>
       </c>
       <c r="D219" s="25" t="s">
         <v>27</v>
@@ -10278,13 +10332,13 @@
     </row>
     <row r="220" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A220" s="25" t="s">
+        <v>728</v>
+      </c>
+      <c r="B220" s="32" t="s">
+        <v>729</v>
+      </c>
+      <c r="C220" s="25" t="s">
         <v>730</v>
-      </c>
-      <c r="B220" s="32" t="s">
-        <v>731</v>
-      </c>
-      <c r="C220" s="25" t="s">
-        <v>732</v>
       </c>
       <c r="D220" s="25" t="s">
         <v>30</v>
@@ -10301,13 +10355,13 @@
     </row>
     <row r="221" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A221" s="25" t="s">
+        <v>731</v>
+      </c>
+      <c r="B221" s="32" t="s">
+        <v>732</v>
+      </c>
+      <c r="C221" s="25" t="s">
         <v>733</v>
-      </c>
-      <c r="B221" s="32" t="s">
-        <v>734</v>
-      </c>
-      <c r="C221" s="25" t="s">
-        <v>735</v>
       </c>
       <c r="D221" s="25" t="s">
         <v>26</v>
@@ -10324,13 +10378,13 @@
     </row>
     <row r="222" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A222" s="25" t="s">
+        <v>734</v>
+      </c>
+      <c r="B222" s="32" t="s">
+        <v>735</v>
+      </c>
+      <c r="C222" s="25" t="s">
         <v>736</v>
-      </c>
-      <c r="B222" s="32" t="s">
-        <v>737</v>
-      </c>
-      <c r="C222" s="25" t="s">
-        <v>738</v>
       </c>
       <c r="D222" s="25" t="s">
         <v>27</v>
@@ -10345,15 +10399,15 @@
         <v>94</v>
       </c>
       <c r="R222" s="27" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
     </row>
     <row r="223" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A223" s="25" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="B223" s="32" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="C223" s="25" t="s">
         <v>81</v>
@@ -10373,13 +10427,13 @@
     </row>
     <row r="224" spans="1:19" ht="136" x14ac:dyDescent="0.2">
       <c r="A224" s="25" t="s">
+        <v>739</v>
+      </c>
+      <c r="B224" s="32" t="s">
+        <v>740</v>
+      </c>
+      <c r="C224" s="25" t="s">
         <v>741</v>
-      </c>
-      <c r="B224" s="32" t="s">
-        <v>742</v>
-      </c>
-      <c r="C224" s="25" t="s">
-        <v>743</v>
       </c>
       <c r="D224" s="25" t="s">
         <v>28</v>
@@ -10396,13 +10450,13 @@
     </row>
     <row r="225" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A225" s="25" t="s">
+        <v>742</v>
+      </c>
+      <c r="B225" s="32" t="s">
+        <v>743</v>
+      </c>
+      <c r="C225" s="25" t="s">
         <v>744</v>
-      </c>
-      <c r="B225" s="32" t="s">
-        <v>745</v>
-      </c>
-      <c r="C225" s="25" t="s">
-        <v>746</v>
       </c>
       <c r="D225" s="25" t="s">
         <v>28</v>
@@ -10419,13 +10473,13 @@
     </row>
     <row r="226" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A226" s="25" t="s">
+        <v>745</v>
+      </c>
+      <c r="B226" s="32" t="s">
+        <v>746</v>
+      </c>
+      <c r="C226" s="25" t="s">
         <v>747</v>
-      </c>
-      <c r="B226" s="32" t="s">
-        <v>748</v>
-      </c>
-      <c r="C226" s="25" t="s">
-        <v>749</v>
       </c>
       <c r="D226" s="25" t="s">
         <v>27</v>
@@ -10442,13 +10496,13 @@
     </row>
     <row r="227" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A227" s="25" t="s">
+        <v>748</v>
+      </c>
+      <c r="B227" s="32" t="s">
+        <v>749</v>
+      </c>
+      <c r="C227" s="25" t="s">
         <v>750</v>
-      </c>
-      <c r="B227" s="32" t="s">
-        <v>751</v>
-      </c>
-      <c r="C227" s="25" t="s">
-        <v>752</v>
       </c>
       <c r="D227" s="25" t="s">
         <v>26</v>
@@ -10465,13 +10519,13 @@
     </row>
     <row r="228" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A228" s="25" t="s">
+        <v>751</v>
+      </c>
+      <c r="B228" s="32" t="s">
+        <v>752</v>
+      </c>
+      <c r="C228" s="25" t="s">
         <v>753</v>
-      </c>
-      <c r="B228" s="32" t="s">
-        <v>754</v>
-      </c>
-      <c r="C228" s="25" t="s">
-        <v>755</v>
       </c>
       <c r="D228" s="25" t="s">
         <v>27</v>
@@ -10486,18 +10540,18 @@
         <v>94</v>
       </c>
       <c r="R228" s="27" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
     </row>
     <row r="229" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A229" s="25" t="s">
+        <v>754</v>
+      </c>
+      <c r="B229" s="32" t="s">
+        <v>755</v>
+      </c>
+      <c r="C229" s="25" t="s">
         <v>756</v>
-      </c>
-      <c r="B229" s="32" t="s">
-        <v>757</v>
-      </c>
-      <c r="C229" s="25" t="s">
-        <v>758</v>
       </c>
       <c r="D229" s="25" t="s">
         <v>26</v>
@@ -10514,13 +10568,13 @@
     </row>
     <row r="230" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A230" s="25" t="s">
+        <v>757</v>
+      </c>
+      <c r="B230" s="32" t="s">
+        <v>758</v>
+      </c>
+      <c r="C230" s="25" t="s">
         <v>759</v>
-      </c>
-      <c r="B230" s="32" t="s">
-        <v>760</v>
-      </c>
-      <c r="C230" s="25" t="s">
-        <v>761</v>
       </c>
       <c r="D230" s="25" t="s">
         <v>30</v>
@@ -10537,13 +10591,13 @@
     </row>
     <row r="231" spans="1:19" ht="119" x14ac:dyDescent="0.2">
       <c r="A231" s="25" t="s">
+        <v>760</v>
+      </c>
+      <c r="B231" s="32" t="s">
+        <v>761</v>
+      </c>
+      <c r="C231" s="25" t="s">
         <v>762</v>
-      </c>
-      <c r="B231" s="32" t="s">
-        <v>763</v>
-      </c>
-      <c r="C231" s="25" t="s">
-        <v>764</v>
       </c>
       <c r="D231" s="25" t="s">
         <v>29</v>
@@ -10560,13 +10614,13 @@
     </row>
     <row r="232" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A232" s="25" t="s">
+        <v>763</v>
+      </c>
+      <c r="B232" s="32" t="s">
+        <v>764</v>
+      </c>
+      <c r="C232" s="25" t="s">
         <v>765</v>
-      </c>
-      <c r="B232" s="32" t="s">
-        <v>766</v>
-      </c>
-      <c r="C232" s="25" t="s">
-        <v>767</v>
       </c>
       <c r="D232" s="25" t="s">
         <v>27</v>
@@ -10583,13 +10637,13 @@
     </row>
     <row r="233" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A233" s="25" t="s">
+        <v>766</v>
+      </c>
+      <c r="B233" s="32" t="s">
+        <v>767</v>
+      </c>
+      <c r="C233" s="25" t="s">
         <v>768</v>
-      </c>
-      <c r="B233" s="32" t="s">
-        <v>769</v>
-      </c>
-      <c r="C233" s="25" t="s">
-        <v>770</v>
       </c>
       <c r="D233" s="25" t="s">
         <v>27</v>
@@ -10606,10 +10660,10 @@
     </row>
     <row r="234" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A234" s="25" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B234" s="32" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="C234" s="25" t="s">
         <v>82</v>
@@ -10632,13 +10686,13 @@
     </row>
     <row r="235" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A235" s="25" t="s">
+        <v>771</v>
+      </c>
+      <c r="B235" s="32" t="s">
+        <v>772</v>
+      </c>
+      <c r="C235" s="25" t="s">
         <v>773</v>
-      </c>
-      <c r="B235" s="32" t="s">
-        <v>774</v>
-      </c>
-      <c r="C235" s="25" t="s">
-        <v>775</v>
       </c>
       <c r="D235" s="25" t="s">
         <v>27</v>
@@ -10653,7 +10707,7 @@
         <v>94</v>
       </c>
       <c r="R235" s="27" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="S235" s="27" t="s">
         <v>68</v>
@@ -10661,13 +10715,13 @@
     </row>
     <row r="236" spans="1:19" ht="85" x14ac:dyDescent="0.2">
       <c r="A236" s="25" t="s">
+        <v>774</v>
+      </c>
+      <c r="B236" s="32" t="s">
+        <v>775</v>
+      </c>
+      <c r="C236" s="25" t="s">
         <v>776</v>
-      </c>
-      <c r="B236" s="32" t="s">
-        <v>777</v>
-      </c>
-      <c r="C236" s="25" t="s">
-        <v>778</v>
       </c>
       <c r="D236" s="25" t="s">
         <v>28</v>
@@ -10684,13 +10738,13 @@
     </row>
     <row r="237" spans="1:19" ht="102" x14ac:dyDescent="0.2">
       <c r="A237" s="25" t="s">
+        <v>777</v>
+      </c>
+      <c r="B237" s="32" t="s">
+        <v>778</v>
+      </c>
+      <c r="C237" s="25" t="s">
         <v>779</v>
-      </c>
-      <c r="B237" s="32" t="s">
-        <v>780</v>
-      </c>
-      <c r="C237" s="25" t="s">
-        <v>781</v>
       </c>
       <c r="D237" s="25" t="s">
         <v>27</v>
@@ -10705,18 +10759,18 @@
         <v>94</v>
       </c>
       <c r="R237" s="27" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
     </row>
     <row r="238" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A238" s="25" t="s">
+        <v>780</v>
+      </c>
+      <c r="B238" s="32" t="s">
+        <v>781</v>
+      </c>
+      <c r="C238" s="25" t="s">
         <v>782</v>
-      </c>
-      <c r="B238" s="32" t="s">
-        <v>783</v>
-      </c>
-      <c r="C238" s="25" t="s">
-        <v>784</v>
       </c>
       <c r="D238" s="25" t="s">
         <v>27</v>
@@ -10733,13 +10787,13 @@
     </row>
     <row r="239" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A239" s="25" t="s">
+        <v>783</v>
+      </c>
+      <c r="B239" s="32" t="s">
+        <v>784</v>
+      </c>
+      <c r="C239" s="25" t="s">
         <v>785</v>
-      </c>
-      <c r="B239" s="32" t="s">
-        <v>786</v>
-      </c>
-      <c r="C239" s="25" t="s">
-        <v>787</v>
       </c>
       <c r="D239" s="25" t="s">
         <v>30</v>
@@ -10756,13 +10810,13 @@
     </row>
     <row r="240" spans="1:19" ht="68" x14ac:dyDescent="0.2">
       <c r="A240" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="B240" s="32" t="s">
+        <v>787</v>
+      </c>
+      <c r="C240" s="25" t="s">
         <v>788</v>
-      </c>
-      <c r="B240" s="32" t="s">
-        <v>789</v>
-      </c>
-      <c r="C240" s="25" t="s">
-        <v>790</v>
       </c>
       <c r="D240" s="25" t="s">
         <v>27</v>
@@ -10782,13 +10836,13 @@
     </row>
     <row r="241" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A241" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="B241" s="32" t="s">
+        <v>790</v>
+      </c>
+      <c r="C241" s="25" t="s">
         <v>791</v>
-      </c>
-      <c r="B241" s="32" t="s">
-        <v>792</v>
-      </c>
-      <c r="C241" s="25" t="s">
-        <v>793</v>
       </c>
       <c r="D241" s="25" t="s">
         <v>28</v>
@@ -10805,13 +10859,13 @@
     </row>
     <row r="242" spans="1:16" ht="68" x14ac:dyDescent="0.2">
       <c r="A242" s="25" t="s">
+        <v>792</v>
+      </c>
+      <c r="B242" s="32" t="s">
+        <v>793</v>
+      </c>
+      <c r="C242" s="25" t="s">
         <v>794</v>
-      </c>
-      <c r="B242" s="32" t="s">
-        <v>795</v>
-      </c>
-      <c r="C242" s="25" t="s">
-        <v>796</v>
       </c>
       <c r="D242" s="25" t="s">
         <v>29</v>
@@ -12176,6 +12230,7 @@
     <hyperlink ref="B24" r:id="rId1" location="ci-c-dev-3" xr:uid="{09A37A58-2BBF-FA48-99E7-8234535ED081}"/>
     <hyperlink ref="B93" r:id="rId2" location="ci-c-found-36" xr:uid="{E9061C6B-069C-4F41-865D-1DCDB9B7CD5D}"/>
     <hyperlink ref="B60" r:id="rId3" location="ci-c-found-6" xr:uid="{33B79C46-F26D-3345-9F9E-821047C0E3E2}"/>
+    <hyperlink ref="B10" r:id="rId4" location="ci-c-conf-5" xr:uid="{F659C0EC-431B-F840-B805-94301197C0AF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -12215,21 +12270,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="48"/>
     </row>
     <row r="2" spans="1:2" ht="82" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="47"/>
-      <c r="B2" s="47"/>
+      <c r="A2" s="48"/>
+      <c r="B2" s="48"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -12291,15 +12346,15 @@
         <v>45</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="153" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>799</v>
-      </c>
-      <c r="B14" s="48" t="s">
-        <v>800</v>
+        <v>797</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>798</v>
       </c>
     </row>
   </sheetData>
@@ -12450,6 +12505,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -12703,15 +12767,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
   <ds:schemaRefs>
@@ -12731,6 +12786,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45EEC221-F5CD-4DEF-B390-EE14E23A8785}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12748,12 +12811,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
requirement approach tracking updates (not displayed)
</commit_message>
<xml_diff>
--- a/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
+++ b/lib/davinci_crd_test_kit/requirements/hl7.fhir.us.davinci-crd_2.2.1_requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karlnaden/GlenViewAssociates/Inferno/source/davinci-crd-test-kit/lib/davinci_crd_test_kit/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{321FB8C7-F3AD-1841-98F0-E9D58B073431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{106BCBB7-FEAF-E945-B1C6-1DC11378FC85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="760" windowWidth="34240" windowHeight="21260" activeTab="1" xr2:uid="{D251129A-65BB-5042-909C-749E11B8C0B0}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="842">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="843">
   <si>
     <r>
       <rPr>
@@ -3882,9 +3882,6 @@
     <t>found-25-B</t>
   </si>
   <si>
-    <t>Limitation: future</t>
-  </si>
-  <si>
     <t>Limitation: what-if not included at this time</t>
   </si>
   <si>
@@ -3916,6 +3913,12 @@
   </si>
   <si>
     <t>NOTE: corrected Appointment with Order -&gt; Appointement without Order</t>
+  </si>
+  <si>
+    <t>Mechanical: demonstrate requests to two different services, one of which requesting a subset of the standard prefetch</t>
+  </si>
+  <si>
+    <t>Mechanical: two different services, each with different prefetch key names and queries.</t>
   </si>
 </sst>
 </file>
@@ -6857,7 +6860,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="34" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:19" ht="51" x14ac:dyDescent="0.2">
       <c r="A80" s="25" t="s">
         <v>829</v>
       </c>
@@ -6880,7 +6883,7 @@
         <v>94</v>
       </c>
       <c r="R80" s="27" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
       <c r="S80" s="27" t="s">
         <v>68</v>
@@ -7024,7 +7027,7 @@
         <v>98</v>
       </c>
       <c r="R86" s="27" t="s">
-        <v>830</v>
+        <v>842</v>
       </c>
       <c r="S86" s="27" t="s">
         <v>68</v>
@@ -7148,7 +7151,7 @@
         <v>94</v>
       </c>
       <c r="R91" s="27" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="92" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -7350,7 +7353,7 @@
         <v>98</v>
       </c>
       <c r="R99" s="27" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="S99" s="27" t="s">
         <v>68</v>
@@ -7860,7 +7863,7 @@
         <v>94</v>
       </c>
       <c r="R120" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S120" s="27" t="s">
         <v>68</v>
@@ -7889,7 +7892,7 @@
         <v>94</v>
       </c>
       <c r="R121" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S121" s="27" t="s">
         <v>68</v>
@@ -7964,7 +7967,7 @@
         <v>94</v>
       </c>
       <c r="R124" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S124" s="27" t="s">
         <v>68</v>
@@ -8016,7 +8019,7 @@
         <v>457</v>
       </c>
       <c r="R126" s="27" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="S126" s="27" t="s">
         <v>68</v>
@@ -8045,7 +8048,7 @@
         <v>94</v>
       </c>
       <c r="R127" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S127" s="27" t="s">
         <v>68</v>
@@ -8097,7 +8100,7 @@
         <v>94</v>
       </c>
       <c r="R129" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S129" s="27" t="s">
         <v>68</v>
@@ -8149,7 +8152,7 @@
         <v>94</v>
       </c>
       <c r="R131" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S131" s="27" t="s">
         <v>68</v>
@@ -8201,7 +8204,7 @@
         <v>457</v>
       </c>
       <c r="R133" s="27" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="S133" s="27" t="s">
         <v>68</v>
@@ -8253,7 +8256,7 @@
         <v>94</v>
       </c>
       <c r="R135" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S135" s="27" t="s">
         <v>68</v>
@@ -8305,7 +8308,7 @@
         <v>94</v>
       </c>
       <c r="R137" s="27" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="S137" s="27" t="s">
         <v>68</v>
@@ -8357,7 +8360,7 @@
         <v>457</v>
       </c>
       <c r="R139" s="27" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="S139" s="27" t="s">
         <v>68</v>
@@ -8435,7 +8438,7 @@
         <v>94</v>
       </c>
       <c r="R142" s="27" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="S142" s="27" t="s">
         <v>68</v>
@@ -8541,7 +8544,7 @@
         <v>520</v>
       </c>
       <c r="C147" s="25" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D147" s="25" t="s">
         <v>27</v>
@@ -8562,7 +8565,7 @@
         <v>68</v>
       </c>
       <c r="U147" s="27" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="148" spans="1:21" ht="170" x14ac:dyDescent="0.2">
@@ -8573,7 +8576,7 @@
         <v>522</v>
       </c>
       <c r="C148" s="25" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D148" s="25" t="s">
         <v>27</v>
@@ -8594,7 +8597,7 @@
         <v>68</v>
       </c>
       <c r="U148" s="27" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="149" spans="1:21" ht="68" x14ac:dyDescent="0.2">
@@ -10393,7 +10396,7 @@
         <v>94</v>
       </c>
       <c r="R222" s="27" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="223" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -10534,7 +10537,7 @@
         <v>94</v>
       </c>
       <c r="R228" s="27" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="229" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -10753,7 +10756,7 @@
         <v>94</v>
       </c>
       <c r="R237" s="27" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="238" spans="1:19" ht="34" x14ac:dyDescent="0.2">
@@ -12225,6 +12228,7 @@
     <hyperlink ref="B93" r:id="rId2" location="ci-c-found-36" xr:uid="{E9061C6B-069C-4F41-865D-1DCDB9B7CD5D}"/>
     <hyperlink ref="B60" r:id="rId3" location="ci-c-found-6" xr:uid="{33B79C46-F26D-3345-9F9E-821047C0E3E2}"/>
     <hyperlink ref="B10" r:id="rId4" location="ci-c-conf-5" xr:uid="{F659C0EC-431B-F840-B805-94301197C0AF}"/>
+    <hyperlink ref="B15" r:id="rId5" location="ci-c-conf-10" xr:uid="{F087E38F-0649-264B-B4E3-ABE51917A024}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
@@ -12499,15 +12503,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EC335ED7BB179244BF94A0DFE64544DC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d3a0f66abe5d2a0564332877ab55d3f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="eebd8b74-b9de-41b2-9247-c010c4973c2b" xmlns:ns3="b7009bbd-f938-489b-a530-f05273710fff" xmlns:ns4="b5a44311-ed64-4a72-909f-c9dc6973bde2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ec7ca2ee893ff8a0f61d4046c6461645" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="eebd8b74-b9de-41b2-9247-c010c4973c2b"/>
@@ -12761,6 +12756,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B0E317-5E0E-4728-AB3F-40F2C2B957FB}">
   <ds:schemaRefs>
@@ -12780,14 +12784,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45EEC221-F5CD-4DEF-B390-EE14E23A8785}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12805,4 +12801,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA84097F-5807-4DCF-92C6-48C9EE26CFB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>